<commit_message>
Curriculum Master: add Subject Area
Maps every subject to one of eight areas (Finance & Accounting,
Economics, Marketing, HR & OB, Information Systems, Analytics,
Strategy, Social Science). The column is in the workbook and
site-data.json, and the Curriculum page shows it with an Area filter.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/E-Logic_BBA_Master_Data_2026-27.xlsx
+++ b/docs/E-Logic_BBA_Master_Data_2026-27.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faculty Master" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curriculum Master'!$A$1:$M$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curriculum Master'!$A$1:$N$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Student Master'!$A$1:$AB$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Faculty Master'!$A$1:$R$57</definedName>
   </definedNames>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -448,14 +448,15 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="48" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -486,40 +487,45 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Subject Area</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Credits</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Sessions per Credit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Total Sessions</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Elective Group</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Evaluation Weighting</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Faculty ID</t>
         </is>
@@ -549,36 +555,41 @@
           <t>Principles of Management</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="I2" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>F018</t>
         </is>
@@ -608,36 +619,41 @@
           <t>Business Economics I (Micro)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="I3" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>F004</t>
         </is>
@@ -667,36 +683,41 @@
           <t>Financial Accounting</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="I4" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>F007</t>
         </is>
@@ -726,36 +747,41 @@
           <t>Business Mathematics</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="I5" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>F013</t>
         </is>
@@ -785,36 +811,41 @@
           <t>Business Communication</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="I6" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>F011</t>
         </is>
@@ -844,36 +875,41 @@
           <t>Digital Productivity Tools</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Information Systems</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="I7" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>F006</t>
         </is>
@@ -903,36 +939,41 @@
           <t>Environmental Studies &amp; Sustainability</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="I8" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>F019</t>
         </is>
@@ -962,36 +1003,41 @@
           <t>Organisational Behaviour</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="I9" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>F005</t>
         </is>
@@ -1021,36 +1067,41 @@
           <t>Business Economics II (Macro)</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="I10" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>F016</t>
         </is>
@@ -1080,36 +1131,41 @@
           <t>Cost &amp; Management Accounting</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="H11" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="I11" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>F014</t>
         </is>
@@ -1139,36 +1195,41 @@
           <t>Business Statistics</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="I12" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>F013</t>
         </is>
@@ -1198,36 +1259,41 @@
           <t>Indian Business Environment</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="H13" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="I13" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>F004</t>
         </is>
@@ -1257,36 +1323,41 @@
           <t>Design Thinking Studio</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="H14" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="I14" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>F012</t>
         </is>
@@ -1316,36 +1387,41 @@
           <t>Community Engagement Project</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="H15" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="I15" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>F019</t>
         </is>
@@ -1375,36 +1451,41 @@
           <t>Marketing Management</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="H16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="I16" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>F003</t>
         </is>
@@ -1434,36 +1515,41 @@
           <t>Financial Management</t>
         </is>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="H17" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="I17" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>F002</t>
         </is>
@@ -1493,36 +1579,41 @@
           <t>Human Resource Management</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="H18" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="I18" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>F017</t>
         </is>
@@ -1552,36 +1643,41 @@
           <t>Business Law</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="H19" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="I19" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>F010</t>
         </is>
@@ -1611,36 +1707,41 @@
           <t>Business Analytics with Excel &amp; Python</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="H20" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="I20" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>F006</t>
         </is>
@@ -1670,36 +1771,41 @@
           <t>Negotiation &amp; Persuasion</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="I21" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>F005</t>
         </is>
@@ -1729,36 +1835,41 @@
           <t>Psychology of Decision Making</t>
         </is>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="H22" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H22" s="2" t="n">
+      <c r="I22" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Open Elective I</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>F016</t>
         </is>
@@ -1788,36 +1899,41 @@
           <t>German Language I</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="H23" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="I23" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Open Elective I</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
         <is>
           <t>F015</t>
         </is>
@@ -1847,36 +1963,41 @@
           <t>Creative Writing for Business</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="2" t="n">
+      <c r="H24" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="I24" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Open Elective I</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>F011</t>
         </is>
@@ -1906,36 +2027,41 @@
           <t>Operations &amp; Supply Chain Management</t>
         </is>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G25" s="2" t="n">
+      <c r="H25" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H25" s="2" t="n">
+      <c r="I25" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>F008</t>
         </is>
@@ -1965,36 +2091,41 @@
           <t>Research Methodology</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="H26" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="I26" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>F013</t>
         </is>
@@ -2024,36 +2155,41 @@
           <t>Consumer Behaviour</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="H27" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H27" s="2" t="n">
+      <c r="I27" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
         <is>
           <t>F009</t>
         </is>
@@ -2083,36 +2219,41 @@
           <t>Entrepreneurship &amp; New Venture Creation</t>
         </is>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="I28" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>F012</t>
         </is>
@@ -2142,36 +2283,41 @@
           <t>Corporate Finance &amp; Banking</t>
         </is>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="H29" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H29" s="2" t="n">
+      <c r="I29" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>F014</t>
         </is>
@@ -2201,36 +2347,41 @@
           <t>Business Simulation Workshop</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="H30" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="I30" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>F008</t>
         </is>
@@ -2260,36 +2411,41 @@
           <t>Digital Marketing Fundamentals</t>
         </is>
       </c>
-      <c r="F31" s="2" t="n">
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="2" t="n">
+      <c r="H31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H31" s="2" t="n">
+      <c r="I31" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>Open Elective II</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>F020</t>
         </is>
@@ -2319,36 +2475,41 @@
           <t>German Language II</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="H32" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H32" s="2" t="n">
+      <c r="I32" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>Open Elective II</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>F015</t>
         </is>
@@ -2378,36 +2539,41 @@
           <t>Behavioural Economics</t>
         </is>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="H33" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="I33" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>Open Elective II</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>F016</t>
         </is>
@@ -2437,36 +2603,41 @@
           <t>Strategic Management</t>
         </is>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="H34" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H34" s="2" t="n">
+      <c r="I34" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>F001</t>
         </is>
@@ -2496,36 +2667,41 @@
           <t>Business Ethics &amp; Corporate Governance</t>
         </is>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="H35" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H35" s="2" t="n">
+      <c r="I35" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>F019</t>
         </is>
@@ -2555,36 +2731,41 @@
           <t>Summer Internship Report &amp; Viva</t>
         </is>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="H36" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H36" s="2" t="n">
+      <c r="I36" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>F012</t>
         </is>
@@ -2614,36 +2795,41 @@
           <t>Leadership Lab</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="H37" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="I37" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M37" s="2" t="inlineStr">
+      <c r="N37" s="2" t="inlineStr">
         <is>
           <t>F017</t>
         </is>
@@ -2673,36 +2859,41 @@
           <t>Sales &amp; Distribution Management</t>
         </is>
       </c>
-      <c r="F38" s="2" t="n">
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G38" s="2" t="n">
+      <c r="H38" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="I38" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M38" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr">
         <is>
           <t>F003</t>
         </is>
@@ -2732,36 +2923,41 @@
           <t>Brand Management</t>
         </is>
       </c>
-      <c r="F39" s="2" t="n">
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G39" s="2" t="n">
+      <c r="H39" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="I39" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr">
         <is>
           <t>F009</t>
         </is>
@@ -2791,36 +2987,41 @@
           <t>Investment Analysis &amp; Portfolio Management</t>
         </is>
       </c>
-      <c r="F40" s="2" t="n">
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G40" s="2" t="n">
+      <c r="H40" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H40" s="2" t="n">
+      <c r="I40" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr">
         <is>
           <t>F002</t>
         </is>
@@ -2850,36 +3051,41 @@
           <t>Financial Markets &amp; Services</t>
         </is>
       </c>
-      <c r="F41" s="2" t="n">
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G41" s="2" t="n">
+      <c r="H41" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H41" s="2" t="n">
+      <c r="I41" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M41" s="2" t="inlineStr">
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>F007</t>
         </is>
@@ -2909,36 +3115,41 @@
           <t>Talent Acquisition &amp; Management</t>
         </is>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G42" s="2" t="n">
+      <c r="H42" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H42" s="2" t="n">
+      <c r="I42" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>Human Resources</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M42" s="2" t="inlineStr">
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>F005</t>
         </is>
@@ -2968,36 +3179,41 @@
           <t>Compensation &amp; Reward Management</t>
         </is>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G43" s="2" t="n">
+      <c r="H43" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H43" s="2" t="n">
+      <c r="I43" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="J43" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>Human Resources</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
+      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M43" s="2" t="inlineStr">
+      <c r="N43" s="2" t="inlineStr">
         <is>
           <t>F017</t>
         </is>
@@ -3027,36 +3243,41 @@
           <t>Data Visualisation &amp; Storytelling</t>
         </is>
       </c>
-      <c r="F44" s="2" t="n">
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G44" s="2" t="n">
+      <c r="H44" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H44" s="2" t="n">
+      <c r="I44" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>Business Analytics</t>
         </is>
       </c>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M44" s="2" t="inlineStr">
+      <c r="N44" s="2" t="inlineStr">
         <is>
           <t>F020</t>
         </is>
@@ -3086,36 +3307,41 @@
           <t>Predictive Analytics for Business</t>
         </is>
       </c>
-      <c r="F45" s="2" t="n">
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G45" s="2" t="n">
+      <c r="H45" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H45" s="2" t="n">
+      <c r="I45" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>Business Analytics</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M45" s="2" t="inlineStr">
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>F006</t>
         </is>
@@ -3145,36 +3371,41 @@
           <t>International Business</t>
         </is>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G46" s="2" t="n">
+      <c r="H46" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H46" s="2" t="n">
+      <c r="I46" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="M46" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M46" s="2" t="inlineStr">
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>F018</t>
         </is>
@@ -3204,36 +3435,41 @@
           <t>Business Taxation (GST &amp; Direct Taxes)</t>
         </is>
       </c>
-      <c r="F47" s="2" t="n">
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G47" s="2" t="n">
+      <c r="H47" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H47" s="2" t="n">
+      <c r="I47" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr">
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L47" s="2" t="inlineStr">
+      <c r="M47" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M47" s="2" t="inlineStr">
+      <c r="N47" s="2" t="inlineStr">
         <is>
           <t>F014</t>
         </is>
@@ -3263,36 +3499,41 @@
           <t>Capstone Consulting Project</t>
         </is>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="H48" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H48" s="2" t="n">
+      <c r="I48" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="M48" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M48" s="2" t="inlineStr">
+      <c r="N48" s="2" t="inlineStr">
         <is>
           <t>F001</t>
         </is>
@@ -3322,36 +3563,41 @@
           <t>Career Readiness Workshop</t>
         </is>
       </c>
-      <c r="F49" s="2" t="n">
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="G49" s="2" t="n">
-        <v>30</v>
       </c>
       <c r="H49" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="I49" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K49" s="2" t="inlineStr">
+      <c r="L49" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L49" s="2" t="inlineStr">
+      <c r="M49" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M49" s="2" t="inlineStr">
+      <c r="N49" s="2" t="inlineStr">
         <is>
           <t>F012</t>
         </is>
@@ -3381,36 +3627,41 @@
           <t>Digital &amp; Social Media Marketing</t>
         </is>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G50" s="2" t="n">
+      <c r="H50" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="I50" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr">
+      <c r="L50" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L50" s="2" t="inlineStr">
+      <c r="M50" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M50" s="2" t="inlineStr">
+      <c r="N50" s="2" t="inlineStr">
         <is>
           <t>F020</t>
         </is>
@@ -3440,36 +3691,41 @@
           <t>Retail Management</t>
         </is>
       </c>
-      <c r="F51" s="2" t="n">
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G51" s="2" t="n">
+      <c r="H51" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H51" s="2" t="n">
+      <c r="I51" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I51" s="2" t="inlineStr">
+      <c r="J51" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr">
+      <c r="K51" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="K51" s="2" t="inlineStr">
+      <c r="L51" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L51" s="2" t="inlineStr">
+      <c r="M51" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M51" s="2" t="inlineStr">
+      <c r="N51" s="2" t="inlineStr">
         <is>
           <t>F009</t>
         </is>
@@ -3499,36 +3755,41 @@
           <t>Corporate Valuation</t>
         </is>
       </c>
-      <c r="F52" s="2" t="n">
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G52" s="2" t="n">
+      <c r="H52" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H52" s="2" t="n">
+      <c r="I52" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="J52" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="K52" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="K52" s="2" t="inlineStr">
+      <c r="L52" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L52" s="2" t="inlineStr">
+      <c r="M52" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M52" s="2" t="inlineStr">
+      <c r="N52" s="2" t="inlineStr">
         <is>
           <t>F002</t>
         </is>
@@ -3558,36 +3819,41 @@
           <t>FinTech &amp; Digital Banking</t>
         </is>
       </c>
-      <c r="F53" s="2" t="n">
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G53" s="2" t="n">
+      <c r="H53" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H53" s="2" t="n">
+      <c r="I53" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="J53" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="K53" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="K53" s="2" t="inlineStr">
+      <c r="L53" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L53" s="2" t="inlineStr">
+      <c r="M53" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M53" s="2" t="inlineStr">
+      <c r="N53" s="2" t="inlineStr">
         <is>
           <t>F007</t>
         </is>
@@ -3617,36 +3883,41 @@
           <t>Learning &amp; Development</t>
         </is>
       </c>
-      <c r="F54" s="2" t="n">
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G54" s="2" t="n">
+      <c r="H54" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H54" s="2" t="n">
+      <c r="I54" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="J54" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="K54" s="2" t="inlineStr">
         <is>
           <t>Human Resources</t>
         </is>
       </c>
-      <c r="K54" s="2" t="inlineStr">
+      <c r="L54" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
+      <c r="M54" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M54" s="2" t="inlineStr">
+      <c r="N54" s="2" t="inlineStr">
         <is>
           <t>F005</t>
         </is>
@@ -3676,36 +3947,41 @@
           <t>Labour Laws &amp; Industrial Relations</t>
         </is>
       </c>
-      <c r="F55" s="2" t="n">
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G55" s="2" t="n">
+      <c r="H55" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H55" s="2" t="n">
+      <c r="I55" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I55" s="2" t="inlineStr">
+      <c r="J55" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="K55" s="2" t="inlineStr">
         <is>
           <t>Human Resources</t>
         </is>
       </c>
-      <c r="K55" s="2" t="inlineStr">
+      <c r="L55" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="L55" s="2" t="inlineStr">
+      <c r="M55" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="M55" s="2" t="inlineStr">
+      <c r="N55" s="2" t="inlineStr">
         <is>
           <t>F010</t>
         </is>
@@ -3735,36 +4011,41 @@
           <t>Machine Learning for Managers</t>
         </is>
       </c>
-      <c r="F56" s="2" t="n">
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G56" s="2" t="n">
+      <c r="H56" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H56" s="2" t="n">
+      <c r="I56" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="I56" s="2" t="inlineStr">
+      <c r="J56" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="K56" s="2" t="inlineStr">
         <is>
           <t>Business Analytics</t>
         </is>
       </c>
-      <c r="K56" s="2" t="inlineStr">
+      <c r="L56" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="L56" s="2" t="inlineStr">
+      <c r="M56" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="M56" s="2" t="inlineStr">
+      <c r="N56" s="2" t="inlineStr">
         <is>
           <t>F013</t>
         </is>
@@ -3794,43 +4075,48 @@
           <t>Business Intelligence with Power BI</t>
         </is>
       </c>
-      <c r="F57" s="2" t="n">
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Information Systems</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G57" s="2" t="n">
+      <c r="H57" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H57" s="2" t="n">
+      <c r="I57" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="I57" s="2" t="inlineStr">
+      <c r="J57" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="K57" s="2" t="inlineStr">
         <is>
           <t>Business Analytics</t>
         </is>
       </c>
-      <c r="K57" s="2" t="inlineStr">
+      <c r="L57" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="L57" s="2" t="inlineStr">
+      <c r="M57" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="M57" s="2" t="inlineStr">
+      <c r="N57" s="2" t="inlineStr">
         <is>
           <t>F006</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M57"/>
+  <autoFilter ref="A1:N57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add section counts to Curriculum Master and Faculty Utilization
Curriculum Master gets "Sections" (sections each subject runs in
2026-27); Faculty Utilization gets "Sections (subject)" so each row
reads as section A of 2. The Curriculum page shows the column and a
"sections running" total.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/E-Logic_BBA_Master_Data_2026-27.xlsx
+++ b/docs/E-Logic_BBA_Master_Data_2026-27.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faculty Utilization" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curriculum Master'!$A$1:$N$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curriculum Master'!$A$1:$O$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Student Master'!$A$1:$AB$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Faculty Master'!$A$1:$H$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Faculty Utilization'!$A$1:$O$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Faculty Utilization'!$A$1:$P$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -455,10 +455,11 @@
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="48" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="48" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -509,25 +510,30 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Sections</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Elective Group</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Assessment</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Evaluation Weighting</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Faculty ID</t>
         </is>
@@ -571,27 +577,30 @@
       <c r="I2" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>F018</t>
         </is>
@@ -635,27 +644,30 @@
       <c r="I3" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>F004</t>
         </is>
@@ -699,27 +711,30 @@
       <c r="I4" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>F007</t>
         </is>
@@ -763,27 +778,30 @@
       <c r="I5" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>F013</t>
         </is>
@@ -827,27 +845,30 @@
       <c r="I6" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>F011</t>
         </is>
@@ -891,27 +912,30 @@
       <c r="I7" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>F006</t>
         </is>
@@ -955,27 +979,30 @@
       <c r="I8" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>F019</t>
         </is>
@@ -1019,27 +1046,30 @@
       <c r="I9" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>F005</t>
         </is>
@@ -1083,27 +1113,30 @@
       <c r="I10" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>F016</t>
         </is>
@@ -1147,27 +1180,30 @@
       <c r="I11" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>F014</t>
         </is>
@@ -1211,27 +1247,30 @@
       <c r="I12" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>F013</t>
         </is>
@@ -1275,27 +1314,30 @@
       <c r="I13" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>F004</t>
         </is>
@@ -1339,27 +1381,30 @@
       <c r="I14" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>F012</t>
         </is>
@@ -1403,27 +1448,30 @@
       <c r="I15" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>F019</t>
         </is>
@@ -1467,27 +1515,30 @@
       <c r="I16" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>F003</t>
         </is>
@@ -1531,27 +1582,30 @@
       <c r="I17" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>F002</t>
         </is>
@@ -1595,27 +1649,30 @@
       <c r="I18" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>F017</t>
         </is>
@@ -1659,27 +1716,30 @@
       <c r="I19" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>F010</t>
         </is>
@@ -1723,27 +1783,30 @@
       <c r="I20" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>F006</t>
         </is>
@@ -1787,27 +1850,30 @@
       <c r="I21" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="O21" s="2" t="inlineStr">
         <is>
           <t>F005</t>
         </is>
@@ -1851,27 +1917,30 @@
       <c r="I22" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Open Elective I</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr">
+      <c r="O22" s="2" t="inlineStr">
         <is>
           <t>F016</t>
         </is>
@@ -1915,27 +1984,30 @@
       <c r="I23" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>Open Elective I</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr">
+      <c r="O23" s="2" t="inlineStr">
         <is>
           <t>F015</t>
         </is>
@@ -1979,27 +2051,30 @@
       <c r="I24" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>Open Elective I</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N24" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>F011</t>
         </is>
@@ -2043,27 +2118,30 @@
       <c r="I25" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr">
+      <c r="O25" s="2" t="inlineStr">
         <is>
           <t>F008</t>
         </is>
@@ -2107,27 +2185,30 @@
       <c r="I26" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>F013</t>
         </is>
@@ -2171,27 +2252,30 @@
       <c r="I27" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr">
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>F009</t>
         </is>
@@ -2235,27 +2319,30 @@
       <c r="I28" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>F012</t>
         </is>
@@ -2299,27 +2386,30 @@
       <c r="I29" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr">
+      <c r="O29" s="2" t="inlineStr">
         <is>
           <t>F014</t>
         </is>
@@ -2363,27 +2453,30 @@
       <c r="I30" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N30" s="2" t="inlineStr">
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>F008</t>
         </is>
@@ -2427,27 +2520,30 @@
       <c r="I31" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>Open Elective II</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N31" s="2" t="inlineStr">
+      <c r="O31" s="2" t="inlineStr">
         <is>
           <t>F020</t>
         </is>
@@ -2491,27 +2587,30 @@
       <c r="I32" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>Open Elective II</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>F015</t>
         </is>
@@ -2555,27 +2654,30 @@
       <c r="I33" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>Open Elective II</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N33" s="2" t="inlineStr">
+      <c r="O33" s="2" t="inlineStr">
         <is>
           <t>F016</t>
         </is>
@@ -2619,27 +2721,30 @@
       <c r="I34" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr">
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>F001</t>
         </is>
@@ -2683,27 +2788,30 @@
       <c r="I35" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N35" s="2" t="inlineStr">
+      <c r="O35" s="2" t="inlineStr">
         <is>
           <t>F019</t>
         </is>
@@ -2747,27 +2855,30 @@
       <c r="I36" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="J36" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N36" s="2" t="inlineStr">
+      <c r="O36" s="2" t="inlineStr">
         <is>
           <t>F012</t>
         </is>
@@ -2811,27 +2922,30 @@
       <c r="I37" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M37" s="2" t="inlineStr">
+      <c r="N37" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N37" s="2" t="inlineStr">
+      <c r="O37" s="2" t="inlineStr">
         <is>
           <t>F017</t>
         </is>
@@ -2875,27 +2989,30 @@
       <c r="I38" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="J38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M38" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N38" s="2" t="inlineStr">
+      <c r="O38" s="2" t="inlineStr">
         <is>
           <t>F003</t>
         </is>
@@ -2939,27 +3056,30 @@
       <c r="I39" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="J39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N39" s="2" t="inlineStr">
+      <c r="O39" s="2" t="inlineStr">
         <is>
           <t>F009</t>
         </is>
@@ -3003,27 +3123,30 @@
       <c r="I40" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="J40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N40" s="2" t="inlineStr">
+      <c r="O40" s="2" t="inlineStr">
         <is>
           <t>F002</t>
         </is>
@@ -3067,27 +3190,30 @@
       <c r="I41" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="J41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M41" s="2" t="inlineStr">
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N41" s="2" t="inlineStr">
+      <c r="O41" s="2" t="inlineStr">
         <is>
           <t>F007</t>
         </is>
@@ -3131,27 +3257,30 @@
       <c r="I42" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="J42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>Human Resources</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M42" s="2" t="inlineStr">
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N42" s="2" t="inlineStr">
+      <c r="O42" s="2" t="inlineStr">
         <is>
           <t>F005</t>
         </is>
@@ -3195,27 +3324,30 @@
       <c r="I43" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="J43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>Human Resources</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
+      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M43" s="2" t="inlineStr">
+      <c r="N43" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N43" s="2" t="inlineStr">
+      <c r="O43" s="2" t="inlineStr">
         <is>
           <t>F017</t>
         </is>
@@ -3259,27 +3391,30 @@
       <c r="I44" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="J44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>Business Analytics</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M44" s="2" t="inlineStr">
+      <c r="N44" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N44" s="2" t="inlineStr">
+      <c r="O44" s="2" t="inlineStr">
         <is>
           <t>F020</t>
         </is>
@@ -3323,27 +3458,30 @@
       <c r="I45" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="J45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>Business Analytics</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M45" s="2" t="inlineStr">
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N45" s="2" t="inlineStr">
+      <c r="O45" s="2" t="inlineStr">
         <is>
           <t>F006</t>
         </is>
@@ -3387,27 +3525,30 @@
       <c r="I46" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="M46" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M46" s="2" t="inlineStr">
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N46" s="2" t="inlineStr">
+      <c r="O46" s="2" t="inlineStr">
         <is>
           <t>F018</t>
         </is>
@@ -3451,27 +3592,30 @@
       <c r="I47" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="J47" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr">
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L47" s="2" t="inlineStr">
+      <c r="M47" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M47" s="2" t="inlineStr">
+      <c r="N47" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N47" s="2" t="inlineStr">
+      <c r="O47" s="2" t="inlineStr">
         <is>
           <t>F014</t>
         </is>
@@ -3515,27 +3659,30 @@
       <c r="I48" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="M48" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M48" s="2" t="inlineStr">
+      <c r="N48" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N48" s="2" t="inlineStr">
+      <c r="O48" s="2" t="inlineStr">
         <is>
           <t>F001</t>
         </is>
@@ -3579,27 +3726,30 @@
       <c r="I49" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="J49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="K49" s="2" t="inlineStr">
+      <c r="L49" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L49" s="2" t="inlineStr">
+      <c r="M49" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M49" s="2" t="inlineStr">
+      <c r="N49" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N49" s="2" t="inlineStr">
+      <c r="O49" s="2" t="inlineStr">
         <is>
           <t>F012</t>
         </is>
@@ -3643,27 +3793,30 @@
       <c r="I50" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="J50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr">
+      <c r="L50" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="L50" s="2" t="inlineStr">
+      <c r="M50" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M50" s="2" t="inlineStr">
+      <c r="N50" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N50" s="2" t="inlineStr">
+      <c r="O50" s="2" t="inlineStr">
         <is>
           <t>F020</t>
         </is>
@@ -3707,27 +3860,30 @@
       <c r="I51" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J51" s="2" t="inlineStr">
+      <c r="J51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K51" s="2" t="inlineStr">
+      <c r="L51" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="L51" s="2" t="inlineStr">
+      <c r="M51" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M51" s="2" t="inlineStr">
+      <c r="N51" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N51" s="2" t="inlineStr">
+      <c r="O51" s="2" t="inlineStr">
         <is>
           <t>F009</t>
         </is>
@@ -3771,27 +3927,30 @@
       <c r="I52" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="J52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K52" s="2" t="inlineStr">
+      <c r="L52" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="L52" s="2" t="inlineStr">
+      <c r="M52" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M52" s="2" t="inlineStr">
+      <c r="N52" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N52" s="2" t="inlineStr">
+      <c r="O52" s="2" t="inlineStr">
         <is>
           <t>F002</t>
         </is>
@@ -3835,27 +3994,30 @@
       <c r="I53" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="J53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K53" s="2" t="inlineStr">
+      <c r="L53" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="L53" s="2" t="inlineStr">
+      <c r="M53" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M53" s="2" t="inlineStr">
+      <c r="N53" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N53" s="2" t="inlineStr">
+      <c r="O53" s="2" t="inlineStr">
         <is>
           <t>F007</t>
         </is>
@@ -3899,27 +4061,30 @@
       <c r="I54" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="J54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K54" s="2" t="inlineStr">
+      <c r="L54" s="2" t="inlineStr">
         <is>
           <t>Human Resources</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
+      <c r="M54" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M54" s="2" t="inlineStr">
+      <c r="N54" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N54" s="2" t="inlineStr">
+      <c r="O54" s="2" t="inlineStr">
         <is>
           <t>F005</t>
         </is>
@@ -3963,27 +4128,30 @@
       <c r="I55" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="J55" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K55" s="2" t="inlineStr">
+      <c r="L55" s="2" t="inlineStr">
         <is>
           <t>Human Resources</t>
         </is>
       </c>
-      <c r="L55" s="2" t="inlineStr">
+      <c r="M55" s="2" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="M55" s="2" t="inlineStr">
+      <c r="N55" s="2" t="inlineStr">
         <is>
           <t>40% internal (quizzes, assignments, mid-term) + 60% end-term exam</t>
         </is>
       </c>
-      <c r="N55" s="2" t="inlineStr">
+      <c r="O55" s="2" t="inlineStr">
         <is>
           <t>F010</t>
         </is>
@@ -4027,27 +4195,30 @@
       <c r="I56" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="J56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K56" s="2" t="inlineStr">
+      <c r="L56" s="2" t="inlineStr">
         <is>
           <t>Business Analytics</t>
         </is>
       </c>
-      <c r="L56" s="2" t="inlineStr">
+      <c r="M56" s="2" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="M56" s="2" t="inlineStr">
+      <c r="N56" s="2" t="inlineStr">
         <is>
           <t>50% internal milestones + 50% final report and viva / presentation</t>
         </is>
       </c>
-      <c r="N56" s="2" t="inlineStr">
+      <c r="O56" s="2" t="inlineStr">
         <is>
           <t>F013</t>
         </is>
@@ -4091,34 +4262,37 @@
       <c r="I57" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="J57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
         <is>
           <t>Elective</t>
         </is>
       </c>
-      <c r="K57" s="2" t="inlineStr">
+      <c r="L57" s="2" t="inlineStr">
         <is>
           <t>Business Analytics</t>
         </is>
       </c>
-      <c r="L57" s="2" t="inlineStr">
+      <c r="M57" s="2" t="inlineStr">
         <is>
           <t>Workshop</t>
         </is>
       </c>
-      <c r="M57" s="2" t="inlineStr">
+      <c r="N57" s="2" t="inlineStr">
         <is>
           <t>100% continuous: studio work, practicals, participation and a final showcase</t>
         </is>
       </c>
-      <c r="N57" s="2" t="inlineStr">
+      <c r="O57" s="2" t="inlineStr">
         <is>
           <t>F006</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N57"/>
+  <autoFilter ref="A1:O57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21586,7 +21760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O91"/>
+  <dimension ref="A1:P91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -21600,10 +21774,11 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="28" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -21664,20 +21839,25 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Sections (subject)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Students</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Credits</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Sessions</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -21738,15 +21918,18 @@
         </is>
       </c>
       <c r="L2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="O2" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -21807,15 +21990,18 @@
         </is>
       </c>
       <c r="L3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="N3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="O3" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -21876,15 +22062,18 @@
         </is>
       </c>
       <c r="L4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="N4" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="O4" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -21945,15 +22134,18 @@
         </is>
       </c>
       <c r="L5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="N5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="O5" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22014,15 +22206,18 @@
         </is>
       </c>
       <c r="L6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="N6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="O6" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22083,15 +22278,18 @@
         </is>
       </c>
       <c r="L7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="N7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="O7" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22152,15 +22350,18 @@
         </is>
       </c>
       <c r="L8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="N8" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="O8" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22221,15 +22422,18 @@
         </is>
       </c>
       <c r="L9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="N9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="O9" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22290,15 +22494,18 @@
         </is>
       </c>
       <c r="L10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="N10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="O10" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22359,15 +22566,18 @@
         </is>
       </c>
       <c r="L11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="N11" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="O11" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22428,15 +22638,18 @@
         </is>
       </c>
       <c r="L12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M12" s="2" t="n">
+      <c r="N12" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="O12" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22497,15 +22710,18 @@
         </is>
       </c>
       <c r="L13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="N13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="O13" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="P13" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22566,15 +22782,18 @@
         </is>
       </c>
       <c r="L14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="N14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="O14" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="P14" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22635,15 +22854,18 @@
         </is>
       </c>
       <c r="L15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="N15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="O15" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="P15" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -22704,15 +22926,18 @@
         </is>
       </c>
       <c r="L16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M16" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="N16" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="O16" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="P16" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -22773,15 +22998,18 @@
         </is>
       </c>
       <c r="L17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M17" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M17" s="2" t="n">
+      <c r="N17" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N17" s="2" t="n">
+      <c r="O17" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -22842,15 +23070,18 @@
         </is>
       </c>
       <c r="L18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="N18" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N18" s="2" t="n">
+      <c r="O18" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="P18" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -22911,15 +23142,18 @@
         </is>
       </c>
       <c r="L19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M19" s="2" t="n">
+      <c r="N19" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N19" s="2" t="n">
+      <c r="O19" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="P19" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -22980,15 +23214,18 @@
         </is>
       </c>
       <c r="L20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M20" s="2" t="n">
+      <c r="N20" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N20" s="2" t="n">
+      <c r="O20" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O20" s="2" t="inlineStr">
+      <c r="P20" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23049,15 +23286,18 @@
         </is>
       </c>
       <c r="L21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M21" s="2" t="n">
+      <c r="N21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N21" s="2" t="n">
+      <c r="O21" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="P21" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23118,15 +23358,18 @@
         </is>
       </c>
       <c r="L22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M22" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M22" s="2" t="n">
+      <c r="N22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N22" s="2" t="n">
+      <c r="O22" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="P22" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23187,15 +23430,18 @@
         </is>
       </c>
       <c r="L23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M23" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M23" s="2" t="n">
+      <c r="N23" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N23" s="2" t="n">
+      <c r="O23" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="P23" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23256,15 +23502,18 @@
         </is>
       </c>
       <c r="L24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M24" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M24" s="2" t="n">
+      <c r="N24" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N24" s="2" t="n">
+      <c r="O24" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O24" s="2" t="inlineStr">
+      <c r="P24" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23325,15 +23574,18 @@
         </is>
       </c>
       <c r="L25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M25" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M25" s="2" t="n">
+      <c r="N25" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N25" s="2" t="n">
+      <c r="O25" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O25" s="2" t="inlineStr">
+      <c r="P25" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23394,15 +23646,18 @@
         </is>
       </c>
       <c r="L26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M26" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M26" s="2" t="n">
+      <c r="N26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N26" s="2" t="n">
+      <c r="O26" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="P26" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23463,15 +23718,18 @@
         </is>
       </c>
       <c r="L27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M27" s="2" t="n">
+      <c r="N27" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N27" s="2" t="n">
+      <c r="O27" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="P27" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23532,15 +23790,18 @@
         </is>
       </c>
       <c r="L28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M28" s="2" t="n">
+      <c r="N28" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N28" s="2" t="n">
+      <c r="O28" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="P28" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23601,15 +23862,18 @@
         </is>
       </c>
       <c r="L29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M29" s="2" t="n">
+      <c r="N29" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N29" s="2" t="n">
+      <c r="O29" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="O29" s="2" t="inlineStr">
+      <c r="P29" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -23670,15 +23934,18 @@
         </is>
       </c>
       <c r="L30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M30" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M30" s="2" t="n">
+      <c r="N30" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N30" s="2" t="n">
+      <c r="O30" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -23739,15 +24006,18 @@
         </is>
       </c>
       <c r="L31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M31" s="2" t="n">
+      <c r="N31" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N31" s="2" t="n">
+      <c r="O31" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O31" s="2" t="inlineStr">
+      <c r="P31" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -23808,15 +24078,18 @@
         </is>
       </c>
       <c r="L32" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M32" s="2" t="n">
+      <c r="N32" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N32" s="2" t="n">
+      <c r="O32" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="P32" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -23877,15 +24150,18 @@
         </is>
       </c>
       <c r="L33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M33" s="2" t="n">
+      <c r="N33" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N33" s="2" t="n">
+      <c r="O33" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O33" s="2" t="inlineStr">
+      <c r="P33" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -23946,15 +24222,18 @@
         </is>
       </c>
       <c r="L34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M34" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M34" s="2" t="n">
+      <c r="N34" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N34" s="2" t="n">
+      <c r="O34" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O34" s="2" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24015,15 +24294,18 @@
         </is>
       </c>
       <c r="L35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M35" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M35" s="2" t="n">
+      <c r="N35" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N35" s="2" t="n">
+      <c r="O35" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O35" s="2" t="inlineStr">
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24084,15 +24366,18 @@
         </is>
       </c>
       <c r="L36" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M36" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M36" s="2" t="n">
+      <c r="N36" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N36" s="2" t="n">
+      <c r="O36" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O36" s="2" t="inlineStr">
+      <c r="P36" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24153,15 +24438,18 @@
         </is>
       </c>
       <c r="L37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M37" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M37" s="2" t="n">
+      <c r="N37" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N37" s="2" t="n">
+      <c r="O37" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O37" s="2" t="inlineStr">
+      <c r="P37" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24222,15 +24510,18 @@
         </is>
       </c>
       <c r="L38" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M38" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M38" s="2" t="n">
+      <c r="N38" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N38" s="2" t="n">
+      <c r="O38" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="O38" s="2" t="inlineStr">
+      <c r="P38" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24291,15 +24582,18 @@
         </is>
       </c>
       <c r="L39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M39" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M39" s="2" t="n">
+      <c r="N39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N39" s="2" t="n">
+      <c r="O39" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="O39" s="2" t="inlineStr">
+      <c r="P39" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24360,15 +24654,18 @@
         </is>
       </c>
       <c r="L40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M40" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M40" s="2" t="n">
+      <c r="N40" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N40" s="2" t="n">
+      <c r="O40" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O40" s="2" t="inlineStr">
+      <c r="P40" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24429,15 +24726,18 @@
         </is>
       </c>
       <c r="L41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M41" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M41" s="2" t="n">
+      <c r="N41" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N41" s="2" t="n">
+      <c r="O41" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O41" s="2" t="inlineStr">
+      <c r="P41" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24498,15 +24798,18 @@
         </is>
       </c>
       <c r="L42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="M42" s="2" t="n">
+      <c r="N42" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N42" s="2" t="n">
+      <c r="O42" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="O42" s="2" t="inlineStr">
+      <c r="P42" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24567,15 +24870,18 @@
         </is>
       </c>
       <c r="L43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M43" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="M43" s="2" t="n">
+      <c r="N43" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N43" s="2" t="n">
+      <c r="O43" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O43" s="2" t="inlineStr">
+      <c r="P43" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24636,15 +24942,18 @@
         </is>
       </c>
       <c r="L44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="M44" s="2" t="n">
+      <c r="N44" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N44" s="2" t="n">
+      <c r="O44" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="O44" s="2" t="inlineStr">
+      <c r="P44" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -24705,15 +25014,18 @@
         </is>
       </c>
       <c r="L45" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M45" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M45" s="2" t="n">
+      <c r="N45" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N45" s="2" t="n">
+      <c r="O45" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O45" s="2" t="inlineStr">
+      <c r="P45" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -24774,15 +25086,18 @@
         </is>
       </c>
       <c r="L46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M46" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M46" s="2" t="n">
+      <c r="N46" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N46" s="2" t="n">
+      <c r="O46" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O46" s="2" t="inlineStr">
+      <c r="P46" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -24843,15 +25158,18 @@
         </is>
       </c>
       <c r="L47" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M47" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M47" s="2" t="n">
+      <c r="N47" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N47" s="2" t="n">
+      <c r="O47" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O47" s="2" t="inlineStr">
+      <c r="P47" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -24912,15 +25230,18 @@
         </is>
       </c>
       <c r="L48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M48" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M48" s="2" t="n">
+      <c r="N48" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N48" s="2" t="n">
+      <c r="O48" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O48" s="2" t="inlineStr">
+      <c r="P48" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -24981,15 +25302,18 @@
         </is>
       </c>
       <c r="L49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M49" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M49" s="2" t="n">
+      <c r="N49" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N49" s="2" t="n">
+      <c r="O49" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O49" s="2" t="inlineStr">
+      <c r="P49" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25050,15 +25374,18 @@
         </is>
       </c>
       <c r="L50" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M50" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M50" s="2" t="n">
+      <c r="N50" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N50" s="2" t="n">
+      <c r="O50" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O50" s="2" t="inlineStr">
+      <c r="P50" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25119,15 +25446,18 @@
         </is>
       </c>
       <c r="L51" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M51" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M51" s="2" t="n">
+      <c r="N51" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N51" s="2" t="n">
+      <c r="O51" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="O51" s="2" t="inlineStr">
+      <c r="P51" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25188,15 +25518,18 @@
         </is>
       </c>
       <c r="L52" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M52" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M52" s="2" t="n">
+      <c r="N52" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N52" s="2" t="n">
+      <c r="O52" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="O52" s="2" t="inlineStr">
+      <c r="P52" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25257,15 +25590,18 @@
         </is>
       </c>
       <c r="L53" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M53" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M53" s="2" t="n">
+      <c r="N53" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N53" s="2" t="n">
+      <c r="O53" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O53" s="2" t="inlineStr">
+      <c r="P53" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25326,15 +25662,18 @@
         </is>
       </c>
       <c r="L54" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M54" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M54" s="2" t="n">
+      <c r="N54" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N54" s="2" t="n">
+      <c r="O54" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O54" s="2" t="inlineStr">
+      <c r="P54" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25395,15 +25734,18 @@
         </is>
       </c>
       <c r="L55" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M55" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M55" s="2" t="n">
+      <c r="N55" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N55" s="2" t="n">
+      <c r="O55" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="O55" s="2" t="inlineStr">
+      <c r="P55" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25464,15 +25806,18 @@
         </is>
       </c>
       <c r="L56" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M56" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M56" s="2" t="n">
+      <c r="N56" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N56" s="2" t="n">
+      <c r="O56" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="O56" s="2" t="inlineStr">
+      <c r="P56" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25533,15 +25878,18 @@
         </is>
       </c>
       <c r="L57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M57" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="M57" s="2" t="n">
+      <c r="N57" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N57" s="2" t="n">
+      <c r="O57" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O57" s="2" t="inlineStr">
+      <c r="P57" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25602,15 +25950,18 @@
         </is>
       </c>
       <c r="L58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M58" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="M58" s="2" t="n">
+      <c r="N58" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N58" s="2" t="n">
+      <c r="O58" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O58" s="2" t="inlineStr">
+      <c r="P58" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25671,15 +26022,18 @@
         </is>
       </c>
       <c r="L59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M59" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M59" s="2" t="n">
+      <c r="N59" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N59" s="2" t="n">
+      <c r="O59" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="O59" s="2" t="inlineStr">
+      <c r="P59" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -25740,15 +26094,18 @@
         </is>
       </c>
       <c r="L60" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M60" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M60" s="2" t="n">
+      <c r="N60" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N60" s="2" t="n">
+      <c r="O60" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O60" s="2" t="inlineStr">
+      <c r="P60" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -25809,15 +26166,18 @@
         </is>
       </c>
       <c r="L61" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M61" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M61" s="2" t="n">
+      <c r="N61" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N61" s="2" t="n">
+      <c r="O61" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O61" s="2" t="inlineStr">
+      <c r="P61" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -25878,15 +26238,18 @@
         </is>
       </c>
       <c r="L62" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M62" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M62" s="2" t="n">
+      <c r="N62" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N62" s="2" t="n">
+      <c r="O62" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O62" s="2" t="inlineStr">
+      <c r="P62" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -25947,15 +26310,18 @@
         </is>
       </c>
       <c r="L63" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M63" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M63" s="2" t="n">
+      <c r="N63" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N63" s="2" t="n">
+      <c r="O63" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O63" s="2" t="inlineStr">
+      <c r="P63" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26016,15 +26382,18 @@
         </is>
       </c>
       <c r="L64" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M64" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M64" s="2" t="n">
+      <c r="N64" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N64" s="2" t="n">
+      <c r="O64" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="O64" s="2" t="inlineStr">
+      <c r="P64" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26085,15 +26454,18 @@
         </is>
       </c>
       <c r="L65" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M65" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M65" s="2" t="n">
+      <c r="N65" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N65" s="2" t="n">
+      <c r="O65" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="O65" s="2" t="inlineStr">
+      <c r="P65" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26154,15 +26526,18 @@
         </is>
       </c>
       <c r="L66" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M66" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M66" s="2" t="n">
+      <c r="N66" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N66" s="2" t="n">
+      <c r="O66" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="O66" s="2" t="inlineStr">
+      <c r="P66" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26223,15 +26598,18 @@
         </is>
       </c>
       <c r="L67" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M67" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M67" s="2" t="n">
+      <c r="N67" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N67" s="2" t="n">
+      <c r="O67" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="O67" s="2" t="inlineStr">
+      <c r="P67" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26292,15 +26670,18 @@
         </is>
       </c>
       <c r="L68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M68" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M68" s="2" t="n">
+      <c r="N68" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N68" s="2" t="n">
+      <c r="O68" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O68" s="2" t="inlineStr">
+      <c r="P68" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26361,15 +26742,18 @@
         </is>
       </c>
       <c r="L69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M69" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M69" s="2" t="n">
+      <c r="N69" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N69" s="2" t="n">
+      <c r="O69" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="O69" s="2" t="inlineStr">
+      <c r="P69" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26430,15 +26814,18 @@
         </is>
       </c>
       <c r="L70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M70" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M70" s="2" t="n">
+      <c r="N70" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N70" s="2" t="n">
+      <c r="O70" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O70" s="2" t="inlineStr">
+      <c r="P70" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26499,15 +26886,18 @@
         </is>
       </c>
       <c r="L71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M71" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M71" s="2" t="n">
+      <c r="N71" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N71" s="2" t="n">
+      <c r="O71" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O71" s="2" t="inlineStr">
+      <c r="P71" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26568,15 +26958,18 @@
         </is>
       </c>
       <c r="L72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M72" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="M72" s="2" t="n">
+      <c r="N72" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N72" s="2" t="n">
+      <c r="O72" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="O72" s="2" t="inlineStr">
+      <c r="P72" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26637,15 +27030,18 @@
         </is>
       </c>
       <c r="L73" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M73" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="M73" s="2" t="n">
+      <c r="N73" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N73" s="2" t="n">
+      <c r="O73" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O73" s="2" t="inlineStr">
+      <c r="P73" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26706,15 +27102,18 @@
         </is>
       </c>
       <c r="L74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M74" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M74" s="2" t="n">
+      <c r="N74" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N74" s="2" t="n">
+      <c r="O74" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="O74" s="2" t="inlineStr">
+      <c r="P74" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26775,15 +27174,18 @@
         </is>
       </c>
       <c r="L75" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M75" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M75" s="2" t="n">
+      <c r="N75" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N75" s="2" t="n">
+      <c r="O75" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="O75" s="2" t="inlineStr">
+      <c r="P75" s="2" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
@@ -26844,15 +27246,18 @@
         </is>
       </c>
       <c r="L76" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M76" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M76" s="2" t="n">
+      <c r="N76" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N76" s="2" t="n">
+      <c r="O76" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O76" s="2" t="inlineStr">
+      <c r="P76" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -26913,15 +27318,18 @@
         </is>
       </c>
       <c r="L77" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M77" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M77" s="2" t="n">
+      <c r="N77" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N77" s="2" t="n">
+      <c r="O77" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O77" s="2" t="inlineStr">
+      <c r="P77" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -26982,15 +27390,18 @@
         </is>
       </c>
       <c r="L78" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M78" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M78" s="2" t="n">
+      <c r="N78" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N78" s="2" t="n">
+      <c r="O78" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O78" s="2" t="inlineStr">
+      <c r="P78" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27051,15 +27462,18 @@
         </is>
       </c>
       <c r="L79" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M79" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M79" s="2" t="n">
+      <c r="N79" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N79" s="2" t="n">
+      <c r="O79" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="O79" s="2" t="inlineStr">
+      <c r="P79" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27120,15 +27534,18 @@
         </is>
       </c>
       <c r="L80" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M80" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M80" s="2" t="n">
+      <c r="N80" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="N80" s="2" t="n">
+      <c r="O80" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="O80" s="2" t="inlineStr">
+      <c r="P80" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27189,15 +27606,18 @@
         </is>
       </c>
       <c r="L81" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M81" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M81" s="2" t="n">
+      <c r="N81" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="N81" s="2" t="n">
+      <c r="O81" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="O81" s="2" t="inlineStr">
+      <c r="P81" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27258,15 +27678,18 @@
         </is>
       </c>
       <c r="L82" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M82" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M82" s="2" t="n">
+      <c r="N82" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N82" s="2" t="n">
+      <c r="O82" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="O82" s="2" t="inlineStr">
+      <c r="P82" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27327,15 +27750,18 @@
         </is>
       </c>
       <c r="L83" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M83" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M83" s="2" t="n">
+      <c r="N83" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N83" s="2" t="n">
+      <c r="O83" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="O83" s="2" t="inlineStr">
+      <c r="P83" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27396,15 +27822,18 @@
         </is>
       </c>
       <c r="L84" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M84" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M84" s="2" t="n">
+      <c r="N84" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N84" s="2" t="n">
+      <c r="O84" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="O84" s="2" t="inlineStr">
+      <c r="P84" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27465,15 +27894,18 @@
         </is>
       </c>
       <c r="L85" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M85" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M85" s="2" t="n">
+      <c r="N85" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N85" s="2" t="n">
+      <c r="O85" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O85" s="2" t="inlineStr">
+      <c r="P85" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27534,15 +27966,18 @@
         </is>
       </c>
       <c r="L86" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M86" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M86" s="2" t="n">
+      <c r="N86" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N86" s="2" t="n">
+      <c r="O86" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="O86" s="2" t="inlineStr">
+      <c r="P86" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27603,15 +28038,18 @@
         </is>
       </c>
       <c r="L87" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M87" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M87" s="2" t="n">
+      <c r="N87" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N87" s="2" t="n">
+      <c r="O87" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O87" s="2" t="inlineStr">
+      <c r="P87" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27672,15 +28110,18 @@
         </is>
       </c>
       <c r="L88" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M88" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="M88" s="2" t="n">
+      <c r="N88" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N88" s="2" t="n">
+      <c r="O88" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="O88" s="2" t="inlineStr">
+      <c r="P88" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27741,15 +28182,18 @@
         </is>
       </c>
       <c r="L89" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M89" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="M89" s="2" t="n">
+      <c r="N89" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N89" s="2" t="n">
+      <c r="O89" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="O89" s="2" t="inlineStr">
+      <c r="P89" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27810,15 +28254,18 @@
         </is>
       </c>
       <c r="L90" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M90" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M90" s="2" t="n">
+      <c r="N90" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N90" s="2" t="n">
+      <c r="O90" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="O90" s="2" t="inlineStr">
+      <c r="P90" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
@@ -27879,22 +28326,25 @@
         </is>
       </c>
       <c r="L91" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M91" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M91" s="2" t="n">
+      <c r="N91" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N91" s="2" t="n">
+      <c r="O91" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="O91" s="2" t="inlineStr">
+      <c r="P91" s="2" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O91"/>
+  <autoFilter ref="A1:P91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Faculty Master: map Area onto the eight subject areas
Each professor's Area now uses the same eight subject areas as the
curriculum, chosen by what they mostly teach. Their own specialism is
kept in a new Specialism column. The Faculty page's Area filter uses
the eight areas, and cards show area and specialism.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/E-Logic_BBA_Master_Data_2026-27.xlsx
+++ b/docs/E-Logic_BBA_Master_Data_2026-27.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curriculum Master'!$A$1:$O$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Student Master'!$A$1:$AB$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Faculty Master'!$A$1:$H$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Faculty Master'!$A$1:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Faculty Utilization'!$A$1:$P$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20892,17 +20892,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -20928,20 +20929,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Specialism</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Qualification</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Experience (years)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Administrative Role</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
@@ -20970,18 +20976,23 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>PhD, Strategic Management</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Dean, School of Business</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>meera.raghavan@elogic.example.edu</t>
         </is>
@@ -21010,18 +21021,23 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>PhD, Finance; CFA charterholder</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Programme Director, BBA</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>arvind.kulkarni@elogic.example.edu</t>
         </is>
@@ -21050,18 +21066,23 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>PhD, Marketing</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>sunita.menon@elogic.example.edu</t>
         </is>
@@ -21090,18 +21111,23 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>PhD, Economics</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>rahul.bhattacharya@elogic.example.edu</t>
         </is>
@@ -21125,23 +21151,28 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>HR &amp; Organisational Behaviour</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>PhD, Organisational Psychology</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Student Welfare &amp; Parent Liaison</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>farah.siddiqui@elogic.example.edu</t>
         </is>
@@ -21165,23 +21196,28 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>Business Analytics</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>MTech (Data Science); PhD pursuing</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>karthik.subramanian@elogic.example.edu</t>
         </is>
@@ -21210,18 +21246,23 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>PhD, Accounting; CA</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Year 2 Coordinator</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>neha.agarwal@elogic.example.edu</t>
         </is>
@@ -21245,23 +21286,28 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>Operations &amp; Supply Chain</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>MBA (Operations); ex-logistics manager</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>joseph.varghese@elogic.example.edu</t>
         </is>
@@ -21290,18 +21336,23 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>PhD, Consumer Behaviour</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Year 3 Coordinator</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>priya.hegde@elogic.example.edu</t>
         </is>
@@ -21325,23 +21376,28 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>Business Law</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>LLM, Corporate Law; practising advocate</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>rohit.malhotra@elogic.example.edu</t>
         </is>
@@ -21365,23 +21421,28 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>Communication</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>PhD, English &amp; Business Communication</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Year 1 Coordinator</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>lakshmi.narayanan@elogic.example.edu</t>
         </is>
@@ -21405,23 +21466,28 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>Entrepreneurship</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>MBA; founder of two start-ups</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Internship &amp; Placement Coordinator</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>ankit.shah@elogic.example.edu</t>
         </is>
@@ -21445,23 +21511,28 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
           <t>Quantitative Methods</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>PhD, Statistics</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>kavya.reddy@elogic.example.edu</t>
         </is>
@@ -21490,18 +21561,23 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
+          <t>Finance &amp; Accounting</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>PhD, Taxation; CA</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Controller of Examinations</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>sanjay.deshmukh@elogic.example.edu</t>
         </is>
@@ -21525,23 +21601,28 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
           <t>Foreign Languages</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>MA, German Studies; Goethe-certified trainer</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>anna.fischer@elogic.example.edu</t>
         </is>
@@ -21570,18 +21651,23 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>PhD, Behavioural Economics</t>
         </is>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>imran.qureshi@elogic.example.edu</t>
         </is>
@@ -21605,23 +21691,28 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>HR &amp; OB</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
           <t>HR &amp; Organisational Behaviour</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>PhD, Human Resource Management</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>pooja.iyer@elogic.example.edu</t>
         </is>
@@ -21645,23 +21736,28 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
           <t>Strategy &amp; International Business</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>MBA; former country head, FMCG</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>vikram.rathore@elogic.example.edu</t>
         </is>
@@ -21685,23 +21781,28 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
+          <t>Social Science</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
           <t>Sustainability &amp; Ethics</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>PhD, Environmental Economics</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>nandini.das@elogic.example.edu</t>
         </is>
@@ -21725,30 +21826,35 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
           <t>Digital Marketing &amp; Analytics</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>MBA; Head of Analytics at a retail firm</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>aditya.kapoor@elogic.example.edu</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H21"/>
+  <autoFilter ref="A1:I21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Faculty Utilization: formula-driven apart from its two inputs
Academic Year, Semester and Faculty ID are now looked up from the
Curriculum Master; Term, Batch and Status are derived from Academic
Year and Semester. Only Subject Code and Section, which define each
row, are typed values. All 2,138 formulas recalculate to their saved
results.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/E-Logic_BBA_Master_Data_2026-27.xlsx
+++ b/docs/E-Logic_BBA_Master_Data_2026-27.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4361" uniqueCount="1212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3911" uniqueCount="1208">
   <si>
     <t>Academic Year</t>
   </si>
@@ -3613,18 +3613,6 @@
   </si>
   <si>
     <t>Status</t>
-  </si>
-  <si>
-    <t>Odd (Jul-Nov 2026)</t>
-  </si>
-  <si>
-    <t>Ongoing</t>
-  </si>
-  <si>
-    <t>Even (Jan-Apr 2027)</t>
-  </si>
-  <si>
-    <t>Upcoming</t>
   </si>
   <si>
     <t>Parameter</t>
@@ -19149,17 +19137,21 @@
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C2" s="2">
+      <c r="A2" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E2,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B2" s="3" t="str">
+        <f>IF(MOD(C2,2)=1,"Odd (Jul-Nov "&amp;LEFT(A2,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A2,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C2" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E2,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>833</v>
+      <c r="D2" s="3" t="str">
+        <f>(LEFT(A2,4)-INT((C2-1)/2))&amp;"-"&amp;RIGHT(LEFT(A2,4)-INT((C2-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>20</v>
@@ -19176,8 +19168,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E2,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>27</v>
+      <c r="I2" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E2,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F018</v>
       </c>
       <c r="J2" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I2,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19218,22 +19211,27 @@
         <f>N2*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T2" s="2" t="s">
-        <v>1196</v>
+      <c r="T2" s="3" t="str">
+        <f>IF(MOD(C2,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C3" s="2">
+      <c r="A3" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E3,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B3" s="3" t="str">
+        <f>IF(MOD(C3,2)=1,"Odd (Jul-Nov "&amp;LEFT(A3,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A3,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C3" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E3,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>833</v>
+      <c r="D3" s="3" t="str">
+        <f>(LEFT(A3,4)-INT((C3-1)/2))&amp;"-"&amp;RIGHT(LEFT(A3,4)-INT((C3-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>20</v>
@@ -19250,8 +19248,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E3,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>27</v>
+      <c r="I3" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E3,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F018</v>
       </c>
       <c r="J3" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I3,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19292,22 +19291,27 @@
         <f>N3*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T3" s="2" t="s">
-        <v>1196</v>
+      <c r="T3" s="3" t="str">
+        <f>IF(MOD(C3,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C4" s="2">
+      <c r="A4" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E4,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B4" s="3" t="str">
+        <f>IF(MOD(C4,2)=1,"Odd (Jul-Nov "&amp;LEFT(A4,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A4,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C4" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E4,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>833</v>
+      <c r="D4" s="3" t="str">
+        <f>(LEFT(A4,4)-INT((C4-1)/2))&amp;"-"&amp;RIGHT(LEFT(A4,4)-INT((C4-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>28</v>
@@ -19324,8 +19328,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E4,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>31</v>
+      <c r="I4" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E4,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F004</v>
       </c>
       <c r="J4" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I4,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19366,22 +19371,27 @@
         <f>N4*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T4" s="2" t="s">
-        <v>1196</v>
+      <c r="T4" s="3" t="str">
+        <f>IF(MOD(C4,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="5" spans="1:20">
-      <c r="A5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C5" s="2">
+      <c r="A5" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E5,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B5" s="3" t="str">
+        <f>IF(MOD(C5,2)=1,"Odd (Jul-Nov "&amp;LEFT(A5,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A5,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C5" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E5,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>833</v>
+      <c r="D5" s="3" t="str">
+        <f>(LEFT(A5,4)-INT((C5-1)/2))&amp;"-"&amp;RIGHT(LEFT(A5,4)-INT((C5-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>28</v>
@@ -19398,8 +19408,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E5,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>31</v>
+      <c r="I5" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E5,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F004</v>
       </c>
       <c r="J5" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I5,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19440,22 +19451,27 @@
         <f>N5*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T5" s="2" t="s">
-        <v>1196</v>
+      <c r="T5" s="3" t="str">
+        <f>IF(MOD(C5,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="6" spans="1:20">
-      <c r="A6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C6" s="2">
+      <c r="A6" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E6,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B6" s="3" t="str">
+        <f>IF(MOD(C6,2)=1,"Odd (Jul-Nov "&amp;LEFT(A6,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A6,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C6" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E6,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>833</v>
+      <c r="D6" s="3" t="str">
+        <f>(LEFT(A6,4)-INT((C6-1)/2))&amp;"-"&amp;RIGHT(LEFT(A6,4)-INT((C6-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>32</v>
@@ -19472,8 +19488,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E6,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>35</v>
+      <c r="I6" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E6,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F007</v>
       </c>
       <c r="J6" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I6,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19514,22 +19531,27 @@
         <f>N6*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T6" s="2" t="s">
-        <v>1196</v>
+      <c r="T6" s="3" t="str">
+        <f>IF(MOD(C6,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C7" s="2">
+      <c r="A7" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E7,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B7" s="3" t="str">
+        <f>IF(MOD(C7,2)=1,"Odd (Jul-Nov "&amp;LEFT(A7,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A7,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C7" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E7,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>833</v>
+      <c r="D7" s="3" t="str">
+        <f>(LEFT(A7,4)-INT((C7-1)/2))&amp;"-"&amp;RIGHT(LEFT(A7,4)-INT((C7-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>32</v>
@@ -19546,8 +19568,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E7,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>35</v>
+      <c r="I7" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E7,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F007</v>
       </c>
       <c r="J7" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I7,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19588,22 +19611,27 @@
         <f>N7*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>1196</v>
+      <c r="T7" s="3" t="str">
+        <f>IF(MOD(C7,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C8" s="2">
+      <c r="A8" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E8,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B8" s="3" t="str">
+        <f>IF(MOD(C8,2)=1,"Odd (Jul-Nov "&amp;LEFT(A8,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A8,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C8" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E8,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>833</v>
+      <c r="D8" s="3" t="str">
+        <f>(LEFT(A8,4)-INT((C8-1)/2))&amp;"-"&amp;RIGHT(LEFT(A8,4)-INT((C8-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>36</v>
@@ -19620,8 +19648,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E8,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I8" s="2" t="s">
-        <v>39</v>
+      <c r="I8" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E8,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F013</v>
       </c>
       <c r="J8" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I8,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19662,22 +19691,27 @@
         <f>N8*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T8" s="2" t="s">
-        <v>1196</v>
+      <c r="T8" s="3" t="str">
+        <f>IF(MOD(C8,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C9" s="2">
+      <c r="A9" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E9,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B9" s="3" t="str">
+        <f>IF(MOD(C9,2)=1,"Odd (Jul-Nov "&amp;LEFT(A9,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A9,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C9" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E9,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>833</v>
+      <c r="D9" s="3" t="str">
+        <f>(LEFT(A9,4)-INT((C9-1)/2))&amp;"-"&amp;RIGHT(LEFT(A9,4)-INT((C9-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>36</v>
@@ -19694,8 +19728,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E9,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>39</v>
+      <c r="I9" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E9,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F013</v>
       </c>
       <c r="J9" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I9,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19736,22 +19771,27 @@
         <f>N9*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T9" s="2" t="s">
-        <v>1196</v>
+      <c r="T9" s="3" t="str">
+        <f>IF(MOD(C9,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="10" spans="1:20">
-      <c r="A10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C10" s="2">
+      <c r="A10" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E10,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B10" s="3" t="str">
+        <f>IF(MOD(C10,2)=1,"Odd (Jul-Nov "&amp;LEFT(A10,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A10,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C10" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E10,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>833</v>
+      <c r="D10" s="3" t="str">
+        <f>(LEFT(A10,4)-INT((C10-1)/2))&amp;"-"&amp;RIGHT(LEFT(A10,4)-INT((C10-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>40</v>
@@ -19768,8 +19808,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E10,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>45</v>
+      <c r="I10" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E10,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F011</v>
       </c>
       <c r="J10" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I10,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19810,22 +19851,27 @@
         <f>N10*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T10" s="2" t="s">
-        <v>1196</v>
+      <c r="T10" s="3" t="str">
+        <f>IF(MOD(C10,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="11" spans="1:20">
-      <c r="A11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C11" s="2">
+      <c r="A11" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E11,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B11" s="3" t="str">
+        <f>IF(MOD(C11,2)=1,"Odd (Jul-Nov "&amp;LEFT(A11,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A11,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C11" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E11,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>833</v>
+      <c r="D11" s="3" t="str">
+        <f>(LEFT(A11,4)-INT((C11-1)/2))&amp;"-"&amp;RIGHT(LEFT(A11,4)-INT((C11-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>40</v>
@@ -19842,8 +19888,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E11,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I11" s="2" t="s">
-        <v>45</v>
+      <c r="I11" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E11,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F011</v>
       </c>
       <c r="J11" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I11,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19884,22 +19931,27 @@
         <f>N11*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T11" s="2" t="s">
-        <v>1196</v>
+      <c r="T11" s="3" t="str">
+        <f>IF(MOD(C11,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="12" spans="1:20">
-      <c r="A12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C12" s="2">
+      <c r="A12" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E12,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B12" s="3" t="str">
+        <f>IF(MOD(C12,2)=1,"Odd (Jul-Nov "&amp;LEFT(A12,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A12,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C12" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E12,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>833</v>
+      <c r="D12" s="3" t="str">
+        <f>(LEFT(A12,4)-INT((C12-1)/2))&amp;"-"&amp;RIGHT(LEFT(A12,4)-INT((C12-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>46</v>
@@ -19916,8 +19968,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E12,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>49</v>
+      <c r="I12" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E12,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F006</v>
       </c>
       <c r="J12" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I12,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -19958,22 +20011,27 @@
         <f>N12*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T12" s="2" t="s">
-        <v>1196</v>
+      <c r="T12" s="3" t="str">
+        <f>IF(MOD(C12,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="13" spans="1:20">
-      <c r="A13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C13" s="2">
+      <c r="A13" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E13,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B13" s="3" t="str">
+        <f>IF(MOD(C13,2)=1,"Odd (Jul-Nov "&amp;LEFT(A13,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A13,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C13" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E13,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>833</v>
+      <c r="D13" s="3" t="str">
+        <f>(LEFT(A13,4)-INT((C13-1)/2))&amp;"-"&amp;RIGHT(LEFT(A13,4)-INT((C13-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>46</v>
@@ -19990,8 +20048,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E13,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I13" s="2" t="s">
-        <v>49</v>
+      <c r="I13" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E13,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F006</v>
       </c>
       <c r="J13" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I13,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20032,22 +20091,27 @@
         <f>N13*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T13" s="2" t="s">
-        <v>1196</v>
+      <c r="T13" s="3" t="str">
+        <f>IF(MOD(C13,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="14" spans="1:20">
-      <c r="A14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C14" s="2">
+      <c r="A14" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E14,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B14" s="3" t="str">
+        <f>IF(MOD(C14,2)=1,"Odd (Jul-Nov "&amp;LEFT(A14,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A14,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C14" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E14,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>833</v>
+      <c r="D14" s="3" t="str">
+        <f>(LEFT(A14,4)-INT((C14-1)/2))&amp;"-"&amp;RIGHT(LEFT(A14,4)-INT((C14-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>50</v>
@@ -20064,8 +20128,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E14,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I14" s="2" t="s">
-        <v>54</v>
+      <c r="I14" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E14,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F019</v>
       </c>
       <c r="J14" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I14,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20106,22 +20171,27 @@
         <f>N14*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T14" s="2" t="s">
-        <v>1196</v>
+      <c r="T14" s="3" t="str">
+        <f>IF(MOD(C14,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="15" spans="1:20">
-      <c r="A15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C15" s="2">
+      <c r="A15" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E15,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B15" s="3" t="str">
+        <f>IF(MOD(C15,2)=1,"Odd (Jul-Nov "&amp;LEFT(A15,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A15,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C15" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E15,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>1</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>833</v>
+      <c r="D15" s="3" t="str">
+        <f>(LEFT(A15,4)-INT((C15-1)/2))&amp;"-"&amp;RIGHT(LEFT(A15,4)-INT((C15-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>50</v>
@@ -20138,8 +20208,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E15,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>54</v>
+      <c r="I15" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E15,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F019</v>
       </c>
       <c r="J15" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I15,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20180,22 +20251,27 @@
         <f>N15*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T15" s="2" t="s">
-        <v>1196</v>
+      <c r="T15" s="3" t="str">
+        <f>IF(MOD(C15,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="16" spans="1:20">
-      <c r="A16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C16" s="2">
+      <c r="A16" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E16,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B16" s="3" t="str">
+        <f>IF(MOD(C16,2)=1,"Odd (Jul-Nov "&amp;LEFT(A16,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A16,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C16" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E16,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>833</v>
+      <c r="D16" s="3" t="str">
+        <f>(LEFT(A16,4)-INT((C16-1)/2))&amp;"-"&amp;RIGHT(LEFT(A16,4)-INT((C16-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>55</v>
@@ -20212,8 +20288,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E16,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>58</v>
+      <c r="I16" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E16,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F005</v>
       </c>
       <c r="J16" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I16,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20254,22 +20331,27 @@
         <f>N16*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T16" s="2" t="s">
-        <v>1198</v>
+      <c r="T16" s="3" t="str">
+        <f>IF(MOD(C16,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="17" spans="1:20">
-      <c r="A17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C17" s="2">
+      <c r="A17" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E17,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B17" s="3" t="str">
+        <f>IF(MOD(C17,2)=1,"Odd (Jul-Nov "&amp;LEFT(A17,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A17,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C17" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E17,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>833</v>
+      <c r="D17" s="3" t="str">
+        <f>(LEFT(A17,4)-INT((C17-1)/2))&amp;"-"&amp;RIGHT(LEFT(A17,4)-INT((C17-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>55</v>
@@ -20286,8 +20368,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E17,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I17" s="2" t="s">
-        <v>58</v>
+      <c r="I17" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E17,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F005</v>
       </c>
       <c r="J17" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I17,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20328,22 +20411,27 @@
         <f>N17*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T17" s="2" t="s">
-        <v>1198</v>
+      <c r="T17" s="3" t="str">
+        <f>IF(MOD(C17,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="18" spans="1:20">
-      <c r="A18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C18" s="2">
+      <c r="A18" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E18,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B18" s="3" t="str">
+        <f>IF(MOD(C18,2)=1,"Odd (Jul-Nov "&amp;LEFT(A18,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A18,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C18" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E18,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>833</v>
+      <c r="D18" s="3" t="str">
+        <f>(LEFT(A18,4)-INT((C18-1)/2))&amp;"-"&amp;RIGHT(LEFT(A18,4)-INT((C18-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>59</v>
@@ -20360,8 +20448,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E18,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I18" s="2" t="s">
-        <v>61</v>
+      <c r="I18" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E18,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F016</v>
       </c>
       <c r="J18" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I18,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20402,22 +20491,27 @@
         <f>N18*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T18" s="2" t="s">
-        <v>1198</v>
+      <c r="T18" s="3" t="str">
+        <f>IF(MOD(C18,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="19" spans="1:20">
-      <c r="A19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C19" s="2">
+      <c r="A19" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E19,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B19" s="3" t="str">
+        <f>IF(MOD(C19,2)=1,"Odd (Jul-Nov "&amp;LEFT(A19,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A19,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C19" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E19,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>833</v>
+      <c r="D19" s="3" t="str">
+        <f>(LEFT(A19,4)-INT((C19-1)/2))&amp;"-"&amp;RIGHT(LEFT(A19,4)-INT((C19-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>59</v>
@@ -20434,8 +20528,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E19,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I19" s="2" t="s">
-        <v>61</v>
+      <c r="I19" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E19,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F016</v>
       </c>
       <c r="J19" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I19,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20476,22 +20571,27 @@
         <f>N19*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T19" s="2" t="s">
-        <v>1198</v>
+      <c r="T19" s="3" t="str">
+        <f>IF(MOD(C19,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="20" spans="1:20">
-      <c r="A20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C20" s="2">
+      <c r="A20" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E20,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B20" s="3" t="str">
+        <f>IF(MOD(C20,2)=1,"Odd (Jul-Nov "&amp;LEFT(A20,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A20,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C20" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E20,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>833</v>
+      <c r="D20" s="3" t="str">
+        <f>(LEFT(A20,4)-INT((C20-1)/2))&amp;"-"&amp;RIGHT(LEFT(A20,4)-INT((C20-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>62</v>
@@ -20508,8 +20608,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E20,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I20" s="2" t="s">
-        <v>64</v>
+      <c r="I20" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E20,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F014</v>
       </c>
       <c r="J20" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I20,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20550,22 +20651,27 @@
         <f>N20*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T20" s="2" t="s">
-        <v>1198</v>
+      <c r="T20" s="3" t="str">
+        <f>IF(MOD(C20,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="21" spans="1:20">
-      <c r="A21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C21" s="2">
+      <c r="A21" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E21,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B21" s="3" t="str">
+        <f>IF(MOD(C21,2)=1,"Odd (Jul-Nov "&amp;LEFT(A21,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A21,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C21" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E21,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>833</v>
+      <c r="D21" s="3" t="str">
+        <f>(LEFT(A21,4)-INT((C21-1)/2))&amp;"-"&amp;RIGHT(LEFT(A21,4)-INT((C21-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>62</v>
@@ -20582,8 +20688,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E21,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I21" s="2" t="s">
-        <v>64</v>
+      <c r="I21" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E21,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F014</v>
       </c>
       <c r="J21" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I21,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20624,22 +20731,27 @@
         <f>N21*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T21" s="2" t="s">
-        <v>1198</v>
+      <c r="T21" s="3" t="str">
+        <f>IF(MOD(C21,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="22" spans="1:20">
-      <c r="A22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C22" s="2">
+      <c r="A22" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E22,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B22" s="3" t="str">
+        <f>IF(MOD(C22,2)=1,"Odd (Jul-Nov "&amp;LEFT(A22,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A22,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C22" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E22,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>833</v>
+      <c r="D22" s="3" t="str">
+        <f>(LEFT(A22,4)-INT((C22-1)/2))&amp;"-"&amp;RIGHT(LEFT(A22,4)-INT((C22-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>65</v>
@@ -20656,8 +20768,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E22,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I22" s="2" t="s">
-        <v>39</v>
+      <c r="I22" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E22,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F013</v>
       </c>
       <c r="J22" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I22,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20698,22 +20811,27 @@
         <f>N22*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T22" s="2" t="s">
-        <v>1198</v>
+      <c r="T22" s="3" t="str">
+        <f>IF(MOD(C22,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="23" spans="1:20">
-      <c r="A23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C23" s="2">
+      <c r="A23" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E23,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B23" s="3" t="str">
+        <f>IF(MOD(C23,2)=1,"Odd (Jul-Nov "&amp;LEFT(A23,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A23,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C23" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E23,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>833</v>
+      <c r="D23" s="3" t="str">
+        <f>(LEFT(A23,4)-INT((C23-1)/2))&amp;"-"&amp;RIGHT(LEFT(A23,4)-INT((C23-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>65</v>
@@ -20730,8 +20848,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E23,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I23" s="2" t="s">
-        <v>39</v>
+      <c r="I23" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E23,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F013</v>
       </c>
       <c r="J23" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I23,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20772,22 +20891,27 @@
         <f>N23*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T23" s="2" t="s">
-        <v>1198</v>
+      <c r="T23" s="3" t="str">
+        <f>IF(MOD(C23,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="24" spans="1:20">
-      <c r="A24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C24" s="2">
+      <c r="A24" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E24,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B24" s="3" t="str">
+        <f>IF(MOD(C24,2)=1,"Odd (Jul-Nov "&amp;LEFT(A24,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A24,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C24" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E24,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>833</v>
+      <c r="D24" s="3" t="str">
+        <f>(LEFT(A24,4)-INT((C24-1)/2))&amp;"-"&amp;RIGHT(LEFT(A24,4)-INT((C24-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>67</v>
@@ -20804,8 +20928,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E24,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I24" s="2" t="s">
-        <v>31</v>
+      <c r="I24" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E24,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F004</v>
       </c>
       <c r="J24" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I24,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20846,22 +20971,27 @@
         <f>N24*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T24" s="2" t="s">
-        <v>1198</v>
+      <c r="T24" s="3" t="str">
+        <f>IF(MOD(C24,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="25" spans="1:20">
-      <c r="A25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C25" s="2">
+      <c r="A25" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E25,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B25" s="3" t="str">
+        <f>IF(MOD(C25,2)=1,"Odd (Jul-Nov "&amp;LEFT(A25,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A25,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C25" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E25,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>833</v>
+      <c r="D25" s="3" t="str">
+        <f>(LEFT(A25,4)-INT((C25-1)/2))&amp;"-"&amp;RIGHT(LEFT(A25,4)-INT((C25-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>67</v>
@@ -20878,8 +21008,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E25,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I25" s="2" t="s">
-        <v>31</v>
+      <c r="I25" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E25,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F004</v>
       </c>
       <c r="J25" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I25,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20920,22 +21051,27 @@
         <f>N25*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T25" s="2" t="s">
-        <v>1198</v>
+      <c r="T25" s="3" t="str">
+        <f>IF(MOD(C25,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="26" spans="1:20">
-      <c r="A26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C26" s="2">
+      <c r="A26" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E26,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B26" s="3" t="str">
+        <f>IF(MOD(C26,2)=1,"Odd (Jul-Nov "&amp;LEFT(A26,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A26,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C26" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E26,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>833</v>
+      <c r="D26" s="3" t="str">
+        <f>(LEFT(A26,4)-INT((C26-1)/2))&amp;"-"&amp;RIGHT(LEFT(A26,4)-INT((C26-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>69</v>
@@ -20952,8 +21088,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E26,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I26" s="2" t="s">
-        <v>71</v>
+      <c r="I26" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E26,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F012</v>
       </c>
       <c r="J26" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I26,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -20994,22 +21131,27 @@
         <f>N26*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T26" s="2" t="s">
-        <v>1198</v>
+      <c r="T26" s="3" t="str">
+        <f>IF(MOD(C26,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="27" spans="1:20">
-      <c r="A27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C27" s="2">
+      <c r="A27" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E27,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B27" s="3" t="str">
+        <f>IF(MOD(C27,2)=1,"Odd (Jul-Nov "&amp;LEFT(A27,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A27,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C27" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E27,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>833</v>
+      <c r="D27" s="3" t="str">
+        <f>(LEFT(A27,4)-INT((C27-1)/2))&amp;"-"&amp;RIGHT(LEFT(A27,4)-INT((C27-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>69</v>
@@ -21026,8 +21168,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E27,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I27" s="2" t="s">
-        <v>71</v>
+      <c r="I27" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E27,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F012</v>
       </c>
       <c r="J27" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I27,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21068,22 +21211,27 @@
         <f>N27*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T27" s="2" t="s">
-        <v>1198</v>
+      <c r="T27" s="3" t="str">
+        <f>IF(MOD(C27,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="28" spans="1:20">
-      <c r="A28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C28" s="2">
+      <c r="A28" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E28,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B28" s="3" t="str">
+        <f>IF(MOD(C28,2)=1,"Odd (Jul-Nov "&amp;LEFT(A28,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A28,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C28" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E28,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>833</v>
+      <c r="D28" s="3" t="str">
+        <f>(LEFT(A28,4)-INT((C28-1)/2))&amp;"-"&amp;RIGHT(LEFT(A28,4)-INT((C28-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>72</v>
@@ -21100,8 +21248,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E28,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I28" s="2" t="s">
-        <v>54</v>
+      <c r="I28" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E28,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F019</v>
       </c>
       <c r="J28" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I28,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21142,22 +21291,27 @@
         <f>N28*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T28" s="2" t="s">
-        <v>1198</v>
+      <c r="T28" s="3" t="str">
+        <f>IF(MOD(C28,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="29" spans="1:20">
-      <c r="A29" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C29" s="2">
+      <c r="A29" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E29,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B29" s="3" t="str">
+        <f>IF(MOD(C29,2)=1,"Odd (Jul-Nov "&amp;LEFT(A29,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A29,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C29" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E29,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>2</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>833</v>
+      <c r="D29" s="3" t="str">
+        <f>(LEFT(A29,4)-INT((C29-1)/2))&amp;"-"&amp;RIGHT(LEFT(A29,4)-INT((C29-1)/2)+3,2)</f>
+        <v>2026-29</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>72</v>
@@ -21174,8 +21328,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E29,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I29" s="2" t="s">
-        <v>54</v>
+      <c r="I29" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E29,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F019</v>
       </c>
       <c r="J29" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I29,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21216,22 +21371,27 @@
         <f>N29*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T29" s="2" t="s">
-        <v>1198</v>
+      <c r="T29" s="3" t="str">
+        <f>IF(MOD(C29,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="30" spans="1:20">
-      <c r="A30" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C30" s="2">
+      <c r="A30" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E30,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B30" s="3" t="str">
+        <f>IF(MOD(C30,2)=1,"Odd (Jul-Nov "&amp;LEFT(A30,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A30,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C30" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E30,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>552</v>
+      <c r="D30" s="3" t="str">
+        <f>(LEFT(A30,4)-INT((C30-1)/2))&amp;"-"&amp;RIGHT(LEFT(A30,4)-INT((C30-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>75</v>
@@ -21248,8 +21408,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E30,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I30" s="2" t="s">
-        <v>78</v>
+      <c r="I30" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E30,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F003</v>
       </c>
       <c r="J30" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I30,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21290,22 +21451,27 @@
         <f>N30*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T30" s="2" t="s">
-        <v>1196</v>
+      <c r="T30" s="3" t="str">
+        <f>IF(MOD(C30,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="31" spans="1:20">
-      <c r="A31" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C31" s="2">
+      <c r="A31" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E31,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B31" s="3" t="str">
+        <f>IF(MOD(C31,2)=1,"Odd (Jul-Nov "&amp;LEFT(A31,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A31,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C31" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E31,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>552</v>
+      <c r="D31" s="3" t="str">
+        <f>(LEFT(A31,4)-INT((C31-1)/2))&amp;"-"&amp;RIGHT(LEFT(A31,4)-INT((C31-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>75</v>
@@ -21322,8 +21488,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E31,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I31" s="2" t="s">
-        <v>78</v>
+      <c r="I31" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E31,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F003</v>
       </c>
       <c r="J31" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I31,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21364,22 +21531,27 @@
         <f>N31*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T31" s="2" t="s">
-        <v>1196</v>
+      <c r="T31" s="3" t="str">
+        <f>IF(MOD(C31,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="32" spans="1:20">
-      <c r="A32" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C32" s="2">
+      <c r="A32" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E32,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B32" s="3" t="str">
+        <f>IF(MOD(C32,2)=1,"Odd (Jul-Nov "&amp;LEFT(A32,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A32,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C32" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E32,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>552</v>
+      <c r="D32" s="3" t="str">
+        <f>(LEFT(A32,4)-INT((C32-1)/2))&amp;"-"&amp;RIGHT(LEFT(A32,4)-INT((C32-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>79</v>
@@ -21396,8 +21568,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E32,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I32" s="2" t="s">
-        <v>81</v>
+      <c r="I32" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E32,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F002</v>
       </c>
       <c r="J32" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I32,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21438,22 +21611,27 @@
         <f>N32*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T32" s="2" t="s">
-        <v>1196</v>
+      <c r="T32" s="3" t="str">
+        <f>IF(MOD(C32,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="33" spans="1:20">
-      <c r="A33" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C33" s="2">
+      <c r="A33" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E33,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B33" s="3" t="str">
+        <f>IF(MOD(C33,2)=1,"Odd (Jul-Nov "&amp;LEFT(A33,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A33,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C33" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E33,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>552</v>
+      <c r="D33" s="3" t="str">
+        <f>(LEFT(A33,4)-INT((C33-1)/2))&amp;"-"&amp;RIGHT(LEFT(A33,4)-INT((C33-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>79</v>
@@ -21470,8 +21648,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E33,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I33" s="2" t="s">
-        <v>81</v>
+      <c r="I33" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E33,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F002</v>
       </c>
       <c r="J33" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I33,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21512,22 +21691,27 @@
         <f>N33*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T33" s="2" t="s">
-        <v>1196</v>
+      <c r="T33" s="3" t="str">
+        <f>IF(MOD(C33,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="34" spans="1:20">
-      <c r="A34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C34" s="2">
+      <c r="A34" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E34,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B34" s="3" t="str">
+        <f>IF(MOD(C34,2)=1,"Odd (Jul-Nov "&amp;LEFT(A34,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A34,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C34" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E34,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>552</v>
+      <c r="D34" s="3" t="str">
+        <f>(LEFT(A34,4)-INT((C34-1)/2))&amp;"-"&amp;RIGHT(LEFT(A34,4)-INT((C34-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>82</v>
@@ -21544,8 +21728,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E34,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I34" s="2" t="s">
-        <v>84</v>
+      <c r="I34" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E34,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F017</v>
       </c>
       <c r="J34" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I34,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21586,22 +21771,27 @@
         <f>N34*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T34" s="2" t="s">
-        <v>1196</v>
+      <c r="T34" s="3" t="str">
+        <f>IF(MOD(C34,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="35" spans="1:20">
-      <c r="A35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C35" s="2">
+      <c r="A35" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E35,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B35" s="3" t="str">
+        <f>IF(MOD(C35,2)=1,"Odd (Jul-Nov "&amp;LEFT(A35,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A35,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C35" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E35,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>552</v>
+      <c r="D35" s="3" t="str">
+        <f>(LEFT(A35,4)-INT((C35-1)/2))&amp;"-"&amp;RIGHT(LEFT(A35,4)-INT((C35-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>82</v>
@@ -21618,8 +21808,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E35,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I35" s="2" t="s">
-        <v>84</v>
+      <c r="I35" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E35,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F017</v>
       </c>
       <c r="J35" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I35,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21660,22 +21851,27 @@
         <f>N35*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T35" s="2" t="s">
-        <v>1196</v>
+      <c r="T35" s="3" t="str">
+        <f>IF(MOD(C35,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="36" spans="1:20">
-      <c r="A36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C36" s="2">
+      <c r="A36" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E36,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B36" s="3" t="str">
+        <f>IF(MOD(C36,2)=1,"Odd (Jul-Nov "&amp;LEFT(A36,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A36,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C36" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E36,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>552</v>
+      <c r="D36" s="3" t="str">
+        <f>(LEFT(A36,4)-INT((C36-1)/2))&amp;"-"&amp;RIGHT(LEFT(A36,4)-INT((C36-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>85</v>
@@ -21692,8 +21888,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E36,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I36" s="2" t="s">
-        <v>87</v>
+      <c r="I36" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E36,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F010</v>
       </c>
       <c r="J36" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I36,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21734,22 +21931,27 @@
         <f>N36*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T36" s="2" t="s">
-        <v>1196</v>
+      <c r="T36" s="3" t="str">
+        <f>IF(MOD(C36,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="37" spans="1:20">
-      <c r="A37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C37" s="2">
+      <c r="A37" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E37,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B37" s="3" t="str">
+        <f>IF(MOD(C37,2)=1,"Odd (Jul-Nov "&amp;LEFT(A37,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A37,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C37" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E37,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>552</v>
+      <c r="D37" s="3" t="str">
+        <f>(LEFT(A37,4)-INT((C37-1)/2))&amp;"-"&amp;RIGHT(LEFT(A37,4)-INT((C37-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>85</v>
@@ -21766,8 +21968,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E37,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I37" s="2" t="s">
-        <v>87</v>
+      <c r="I37" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E37,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F010</v>
       </c>
       <c r="J37" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I37,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21808,22 +22011,27 @@
         <f>N37*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T37" s="2" t="s">
-        <v>1196</v>
+      <c r="T37" s="3" t="str">
+        <f>IF(MOD(C37,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="38" spans="1:20">
-      <c r="A38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C38" s="2">
+      <c r="A38" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E38,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B38" s="3" t="str">
+        <f>IF(MOD(C38,2)=1,"Odd (Jul-Nov "&amp;LEFT(A38,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A38,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C38" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E38,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>552</v>
+      <c r="D38" s="3" t="str">
+        <f>(LEFT(A38,4)-INT((C38-1)/2))&amp;"-"&amp;RIGHT(LEFT(A38,4)-INT((C38-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>88</v>
@@ -21840,8 +22048,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E38,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I38" s="2" t="s">
-        <v>49</v>
+      <c r="I38" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E38,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F006</v>
       </c>
       <c r="J38" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I38,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21882,22 +22091,27 @@
         <f>N38*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T38" s="2" t="s">
-        <v>1196</v>
+      <c r="T38" s="3" t="str">
+        <f>IF(MOD(C38,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="39" spans="1:20">
-      <c r="A39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C39" s="2">
+      <c r="A39" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E39,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B39" s="3" t="str">
+        <f>IF(MOD(C39,2)=1,"Odd (Jul-Nov "&amp;LEFT(A39,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A39,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C39" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E39,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>552</v>
+      <c r="D39" s="3" t="str">
+        <f>(LEFT(A39,4)-INT((C39-1)/2))&amp;"-"&amp;RIGHT(LEFT(A39,4)-INT((C39-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>88</v>
@@ -21914,8 +22128,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E39,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I39" s="2" t="s">
-        <v>49</v>
+      <c r="I39" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E39,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F006</v>
       </c>
       <c r="J39" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I39,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -21956,22 +22171,27 @@
         <f>N39*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T39" s="2" t="s">
-        <v>1196</v>
+      <c r="T39" s="3" t="str">
+        <f>IF(MOD(C39,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="40" spans="1:20">
-      <c r="A40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C40" s="2">
+      <c r="A40" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E40,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B40" s="3" t="str">
+        <f>IF(MOD(C40,2)=1,"Odd (Jul-Nov "&amp;LEFT(A40,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A40,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C40" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E40,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>552</v>
+      <c r="D40" s="3" t="str">
+        <f>(LEFT(A40,4)-INT((C40-1)/2))&amp;"-"&amp;RIGHT(LEFT(A40,4)-INT((C40-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>90</v>
@@ -21988,8 +22208,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E40,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I40" s="2" t="s">
-        <v>58</v>
+      <c r="I40" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E40,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F005</v>
       </c>
       <c r="J40" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I40,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22030,22 +22251,27 @@
         <f>N40*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T40" s="2" t="s">
-        <v>1196</v>
+      <c r="T40" s="3" t="str">
+        <f>IF(MOD(C40,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="41" spans="1:20">
-      <c r="A41" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C41" s="2">
+      <c r="A41" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E41,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B41" s="3" t="str">
+        <f>IF(MOD(C41,2)=1,"Odd (Jul-Nov "&amp;LEFT(A41,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A41,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C41" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E41,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>552</v>
+      <c r="D41" s="3" t="str">
+        <f>(LEFT(A41,4)-INT((C41-1)/2))&amp;"-"&amp;RIGHT(LEFT(A41,4)-INT((C41-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>90</v>
@@ -22062,8 +22288,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E41,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I41" s="2" t="s">
-        <v>58</v>
+      <c r="I41" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E41,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F005</v>
       </c>
       <c r="J41" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I41,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22104,22 +22331,27 @@
         <f>N41*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T41" s="2" t="s">
-        <v>1196</v>
+      <c r="T41" s="3" t="str">
+        <f>IF(MOD(C41,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="42" spans="1:20">
-      <c r="A42" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C42" s="2">
+      <c r="A42" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E42,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B42" s="3" t="str">
+        <f>IF(MOD(C42,2)=1,"Odd (Jul-Nov "&amp;LEFT(A42,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A42,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C42" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E42,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>552</v>
+      <c r="D42" s="3" t="str">
+        <f>(LEFT(A42,4)-INT((C42-1)/2))&amp;"-"&amp;RIGHT(LEFT(A42,4)-INT((C42-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>92</v>
@@ -22136,8 +22368,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E42,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I42" s="2" t="s">
-        <v>61</v>
+      <c r="I42" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E42,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F016</v>
       </c>
       <c r="J42" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I42,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22178,22 +22411,27 @@
         <f>N42*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T42" s="2" t="s">
-        <v>1196</v>
+      <c r="T42" s="3" t="str">
+        <f>IF(MOD(C42,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="43" spans="1:20">
-      <c r="A43" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C43" s="2">
+      <c r="A43" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E43,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B43" s="3" t="str">
+        <f>IF(MOD(C43,2)=1,"Odd (Jul-Nov "&amp;LEFT(A43,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A43,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C43" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E43,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>552</v>
+      <c r="D43" s="3" t="str">
+        <f>(LEFT(A43,4)-INT((C43-1)/2))&amp;"-"&amp;RIGHT(LEFT(A43,4)-INT((C43-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>96</v>
@@ -22210,8 +22448,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E43,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I43" s="2" t="s">
-        <v>98</v>
+      <c r="I43" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E43,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F015</v>
       </c>
       <c r="J43" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I43,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22252,22 +22491,27 @@
         <f>N43*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T43" s="2" t="s">
-        <v>1196</v>
+      <c r="T43" s="3" t="str">
+        <f>IF(MOD(C43,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="44" spans="1:20">
-      <c r="A44" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C44" s="2">
+      <c r="A44" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E44,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B44" s="3" t="str">
+        <f>IF(MOD(C44,2)=1,"Odd (Jul-Nov "&amp;LEFT(A44,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A44,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C44" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E44,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>3</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>552</v>
+      <c r="D44" s="3" t="str">
+        <f>(LEFT(A44,4)-INT((C44-1)/2))&amp;"-"&amp;RIGHT(LEFT(A44,4)-INT((C44-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>99</v>
@@ -22284,8 +22528,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E44,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I44" s="2" t="s">
-        <v>45</v>
+      <c r="I44" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E44,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F011</v>
       </c>
       <c r="J44" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I44,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22326,22 +22571,27 @@
         <f>N44*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T44" s="2" t="s">
-        <v>1196</v>
+      <c r="T44" s="3" t="str">
+        <f>IF(MOD(C44,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="45" spans="1:20">
-      <c r="A45" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C45" s="2">
+      <c r="A45" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E45,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B45" s="3" t="str">
+        <f>IF(MOD(C45,2)=1,"Odd (Jul-Nov "&amp;LEFT(A45,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A45,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C45" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E45,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>552</v>
+      <c r="D45" s="3" t="str">
+        <f>(LEFT(A45,4)-INT((C45-1)/2))&amp;"-"&amp;RIGHT(LEFT(A45,4)-INT((C45-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>101</v>
@@ -22358,8 +22608,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E45,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I45" s="2" t="s">
-        <v>103</v>
+      <c r="I45" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E45,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F008</v>
       </c>
       <c r="J45" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I45,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22400,22 +22651,27 @@
         <f>N45*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T45" s="2" t="s">
-        <v>1198</v>
+      <c r="T45" s="3" t="str">
+        <f>IF(MOD(C45,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="46" spans="1:20">
-      <c r="A46" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C46" s="2">
+      <c r="A46" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E46,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B46" s="3" t="str">
+        <f>IF(MOD(C46,2)=1,"Odd (Jul-Nov "&amp;LEFT(A46,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A46,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C46" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E46,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>552</v>
+      <c r="D46" s="3" t="str">
+        <f>(LEFT(A46,4)-INT((C46-1)/2))&amp;"-"&amp;RIGHT(LEFT(A46,4)-INT((C46-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>101</v>
@@ -22432,8 +22688,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E46,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I46" s="2" t="s">
-        <v>103</v>
+      <c r="I46" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E46,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F008</v>
       </c>
       <c r="J46" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I46,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22474,22 +22731,27 @@
         <f>N46*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T46" s="2" t="s">
-        <v>1198</v>
+      <c r="T46" s="3" t="str">
+        <f>IF(MOD(C46,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="47" spans="1:20">
-      <c r="A47" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C47" s="2">
+      <c r="A47" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E47,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B47" s="3" t="str">
+        <f>IF(MOD(C47,2)=1,"Odd (Jul-Nov "&amp;LEFT(A47,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A47,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C47" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E47,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D47" s="2" t="s">
-        <v>552</v>
+      <c r="D47" s="3" t="str">
+        <f>(LEFT(A47,4)-INT((C47-1)/2))&amp;"-"&amp;RIGHT(LEFT(A47,4)-INT((C47-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>104</v>
@@ -22506,8 +22768,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E47,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I47" s="2" t="s">
-        <v>39</v>
+      <c r="I47" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E47,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F013</v>
       </c>
       <c r="J47" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I47,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22548,22 +22811,27 @@
         <f>N47*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T47" s="2" t="s">
-        <v>1198</v>
+      <c r="T47" s="3" t="str">
+        <f>IF(MOD(C47,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="48" spans="1:20">
-      <c r="A48" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C48" s="2">
+      <c r="A48" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E48,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B48" s="3" t="str">
+        <f>IF(MOD(C48,2)=1,"Odd (Jul-Nov "&amp;LEFT(A48,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A48,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C48" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E48,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>552</v>
+      <c r="D48" s="3" t="str">
+        <f>(LEFT(A48,4)-INT((C48-1)/2))&amp;"-"&amp;RIGHT(LEFT(A48,4)-INT((C48-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>104</v>
@@ -22580,8 +22848,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E48,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I48" s="2" t="s">
-        <v>39</v>
+      <c r="I48" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E48,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F013</v>
       </c>
       <c r="J48" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I48,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22622,22 +22891,27 @@
         <f>N48*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T48" s="2" t="s">
-        <v>1198</v>
+      <c r="T48" s="3" t="str">
+        <f>IF(MOD(C48,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="49" spans="1:20">
-      <c r="A49" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C49" s="2">
+      <c r="A49" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E49,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B49" s="3" t="str">
+        <f>IF(MOD(C49,2)=1,"Odd (Jul-Nov "&amp;LEFT(A49,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A49,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C49" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E49,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>552</v>
+      <c r="D49" s="3" t="str">
+        <f>(LEFT(A49,4)-INT((C49-1)/2))&amp;"-"&amp;RIGHT(LEFT(A49,4)-INT((C49-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>106</v>
@@ -22654,8 +22928,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E49,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I49" s="2" t="s">
-        <v>108</v>
+      <c r="I49" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E49,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F009</v>
       </c>
       <c r="J49" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I49,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22696,22 +22971,27 @@
         <f>N49*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T49" s="2" t="s">
-        <v>1198</v>
+      <c r="T49" s="3" t="str">
+        <f>IF(MOD(C49,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="50" spans="1:20">
-      <c r="A50" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C50" s="2">
+      <c r="A50" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E50,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B50" s="3" t="str">
+        <f>IF(MOD(C50,2)=1,"Odd (Jul-Nov "&amp;LEFT(A50,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A50,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C50" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E50,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>552</v>
+      <c r="D50" s="3" t="str">
+        <f>(LEFT(A50,4)-INT((C50-1)/2))&amp;"-"&amp;RIGHT(LEFT(A50,4)-INT((C50-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>106</v>
@@ -22728,8 +23008,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E50,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I50" s="2" t="s">
-        <v>108</v>
+      <c r="I50" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E50,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F009</v>
       </c>
       <c r="J50" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I50,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22770,22 +23051,27 @@
         <f>N50*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T50" s="2" t="s">
-        <v>1198</v>
+      <c r="T50" s="3" t="str">
+        <f>IF(MOD(C50,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="51" spans="1:20">
-      <c r="A51" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C51" s="2">
+      <c r="A51" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E51,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B51" s="3" t="str">
+        <f>IF(MOD(C51,2)=1,"Odd (Jul-Nov "&amp;LEFT(A51,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A51,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C51" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E51,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D51" s="2" t="s">
-        <v>552</v>
+      <c r="D51" s="3" t="str">
+        <f>(LEFT(A51,4)-INT((C51-1)/2))&amp;"-"&amp;RIGHT(LEFT(A51,4)-INT((C51-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>109</v>
@@ -22802,8 +23088,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E51,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I51" s="2" t="s">
-        <v>71</v>
+      <c r="I51" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E51,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F012</v>
       </c>
       <c r="J51" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I51,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22844,22 +23131,27 @@
         <f>N51*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T51" s="2" t="s">
-        <v>1198</v>
+      <c r="T51" s="3" t="str">
+        <f>IF(MOD(C51,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="52" spans="1:20">
-      <c r="A52" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C52" s="2">
+      <c r="A52" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E52,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B52" s="3" t="str">
+        <f>IF(MOD(C52,2)=1,"Odd (Jul-Nov "&amp;LEFT(A52,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A52,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C52" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E52,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D52" s="2" t="s">
-        <v>552</v>
+      <c r="D52" s="3" t="str">
+        <f>(LEFT(A52,4)-INT((C52-1)/2))&amp;"-"&amp;RIGHT(LEFT(A52,4)-INT((C52-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>109</v>
@@ -22876,8 +23168,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E52,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I52" s="2" t="s">
-        <v>71</v>
+      <c r="I52" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E52,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F012</v>
       </c>
       <c r="J52" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I52,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22918,22 +23211,27 @@
         <f>N52*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T52" s="2" t="s">
-        <v>1198</v>
+      <c r="T52" s="3" t="str">
+        <f>IF(MOD(C52,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="53" spans="1:20">
-      <c r="A53" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C53" s="2">
+      <c r="A53" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E53,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B53" s="3" t="str">
+        <f>IF(MOD(C53,2)=1,"Odd (Jul-Nov "&amp;LEFT(A53,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A53,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C53" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E53,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D53" s="2" t="s">
-        <v>552</v>
+      <c r="D53" s="3" t="str">
+        <f>(LEFT(A53,4)-INT((C53-1)/2))&amp;"-"&amp;RIGHT(LEFT(A53,4)-INT((C53-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>111</v>
@@ -22950,8 +23248,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E53,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I53" s="2" t="s">
-        <v>64</v>
+      <c r="I53" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E53,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F014</v>
       </c>
       <c r="J53" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I53,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -22992,22 +23291,27 @@
         <f>N53*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T53" s="2" t="s">
-        <v>1198</v>
+      <c r="T53" s="3" t="str">
+        <f>IF(MOD(C53,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="54" spans="1:20">
-      <c r="A54" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C54" s="2">
+      <c r="A54" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E54,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B54" s="3" t="str">
+        <f>IF(MOD(C54,2)=1,"Odd (Jul-Nov "&amp;LEFT(A54,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A54,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C54" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E54,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>552</v>
+      <c r="D54" s="3" t="str">
+        <f>(LEFT(A54,4)-INT((C54-1)/2))&amp;"-"&amp;RIGHT(LEFT(A54,4)-INT((C54-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>111</v>
@@ -23024,8 +23328,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E54,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I54" s="2" t="s">
-        <v>64</v>
+      <c r="I54" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E54,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F014</v>
       </c>
       <c r="J54" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I54,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23066,22 +23371,27 @@
         <f>N54*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T54" s="2" t="s">
-        <v>1198</v>
+      <c r="T54" s="3" t="str">
+        <f>IF(MOD(C54,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="55" spans="1:20">
-      <c r="A55" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C55" s="2">
+      <c r="A55" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E55,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B55" s="3" t="str">
+        <f>IF(MOD(C55,2)=1,"Odd (Jul-Nov "&amp;LEFT(A55,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A55,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C55" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E55,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D55" s="2" t="s">
-        <v>552</v>
+      <c r="D55" s="3" t="str">
+        <f>(LEFT(A55,4)-INT((C55-1)/2))&amp;"-"&amp;RIGHT(LEFT(A55,4)-INT((C55-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>113</v>
@@ -23098,8 +23408,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E55,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I55" s="2" t="s">
-        <v>103</v>
+      <c r="I55" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E55,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F008</v>
       </c>
       <c r="J55" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I55,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23140,22 +23451,27 @@
         <f>N55*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T55" s="2" t="s">
-        <v>1198</v>
+      <c r="T55" s="3" t="str">
+        <f>IF(MOD(C55,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="56" spans="1:20">
-      <c r="A56" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C56" s="2">
+      <c r="A56" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E56,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B56" s="3" t="str">
+        <f>IF(MOD(C56,2)=1,"Odd (Jul-Nov "&amp;LEFT(A56,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A56,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C56" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E56,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>552</v>
+      <c r="D56" s="3" t="str">
+        <f>(LEFT(A56,4)-INT((C56-1)/2))&amp;"-"&amp;RIGHT(LEFT(A56,4)-INT((C56-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>113</v>
@@ -23172,8 +23488,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E56,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I56" s="2" t="s">
-        <v>103</v>
+      <c r="I56" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E56,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F008</v>
       </c>
       <c r="J56" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I56,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23214,22 +23531,27 @@
         <f>N56*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T56" s="2" t="s">
-        <v>1198</v>
+      <c r="T56" s="3" t="str">
+        <f>IF(MOD(C56,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="57" spans="1:20">
-      <c r="A57" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C57" s="2">
+      <c r="A57" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E57,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B57" s="3" t="str">
+        <f>IF(MOD(C57,2)=1,"Odd (Jul-Nov "&amp;LEFT(A57,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A57,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C57" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E57,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>552</v>
+      <c r="D57" s="3" t="str">
+        <f>(LEFT(A57,4)-INT((C57-1)/2))&amp;"-"&amp;RIGHT(LEFT(A57,4)-INT((C57-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>115</v>
@@ -23246,8 +23568,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E57,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I57" s="2" t="s">
-        <v>118</v>
+      <c r="I57" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E57,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F020</v>
       </c>
       <c r="J57" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I57,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23288,22 +23611,27 @@
         <f>N57*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T57" s="2" t="s">
-        <v>1198</v>
+      <c r="T57" s="3" t="str">
+        <f>IF(MOD(C57,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="58" spans="1:20">
-      <c r="A58" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C58" s="2">
+      <c r="A58" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E58,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B58" s="3" t="str">
+        <f>IF(MOD(C58,2)=1,"Odd (Jul-Nov "&amp;LEFT(A58,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A58,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C58" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E58,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D58" s="2" t="s">
-        <v>552</v>
+      <c r="D58" s="3" t="str">
+        <f>(LEFT(A58,4)-INT((C58-1)/2))&amp;"-"&amp;RIGHT(LEFT(A58,4)-INT((C58-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>119</v>
@@ -23320,8 +23648,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E58,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I58" s="2" t="s">
-        <v>98</v>
+      <c r="I58" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E58,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F015</v>
       </c>
       <c r="J58" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I58,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23362,22 +23691,27 @@
         <f>N58*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T58" s="2" t="s">
-        <v>1198</v>
+      <c r="T58" s="3" t="str">
+        <f>IF(MOD(C58,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="59" spans="1:20">
-      <c r="A59" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C59" s="2">
+      <c r="A59" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E59,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B59" s="3" t="str">
+        <f>IF(MOD(C59,2)=1,"Odd (Jul-Nov "&amp;LEFT(A59,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A59,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C59" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E59,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>4</v>
       </c>
-      <c r="D59" s="2" t="s">
-        <v>552</v>
+      <c r="D59" s="3" t="str">
+        <f>(LEFT(A59,4)-INT((C59-1)/2))&amp;"-"&amp;RIGHT(LEFT(A59,4)-INT((C59-1)/2)+3,2)</f>
+        <v>2025-28</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>121</v>
@@ -23394,8 +23728,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E59,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I59" s="2" t="s">
-        <v>61</v>
+      <c r="I59" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E59,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F016</v>
       </c>
       <c r="J59" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I59,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23436,22 +23771,27 @@
         <f>N59*FacultyCreditHoursPerCredit</f>
         <v>30</v>
       </c>
-      <c r="T59" s="2" t="s">
-        <v>1198</v>
+      <c r="T59" s="3" t="str">
+        <f>IF(MOD(C59,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="60" spans="1:20">
-      <c r="A60" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C60" s="2">
+      <c r="A60" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E60,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B60" s="3" t="str">
+        <f>IF(MOD(C60,2)=1,"Odd (Jul-Nov "&amp;LEFT(A60,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A60,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C60" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E60,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D60" s="2" t="s">
-        <v>208</v>
+      <c r="D60" s="3" t="str">
+        <f>(LEFT(A60,4)-INT((C60-1)/2))&amp;"-"&amp;RIGHT(LEFT(A60,4)-INT((C60-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>124</v>
@@ -23468,8 +23808,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E60,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I60" s="2" t="s">
-        <v>126</v>
+      <c r="I60" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E60,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F001</v>
       </c>
       <c r="J60" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I60,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23510,22 +23851,27 @@
         <f>N60*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T60" s="2" t="s">
-        <v>1196</v>
+      <c r="T60" s="3" t="str">
+        <f>IF(MOD(C60,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="61" spans="1:20">
-      <c r="A61" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C61" s="2">
+      <c r="A61" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E61,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B61" s="3" t="str">
+        <f>IF(MOD(C61,2)=1,"Odd (Jul-Nov "&amp;LEFT(A61,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A61,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C61" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E61,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D61" s="2" t="s">
-        <v>208</v>
+      <c r="D61" s="3" t="str">
+        <f>(LEFT(A61,4)-INT((C61-1)/2))&amp;"-"&amp;RIGHT(LEFT(A61,4)-INT((C61-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>124</v>
@@ -23542,8 +23888,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E61,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I61" s="2" t="s">
-        <v>126</v>
+      <c r="I61" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E61,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F001</v>
       </c>
       <c r="J61" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I61,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23584,22 +23931,27 @@
         <f>N61*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T61" s="2" t="s">
-        <v>1196</v>
+      <c r="T61" s="3" t="str">
+        <f>IF(MOD(C61,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="62" spans="1:20">
-      <c r="A62" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C62" s="2">
+      <c r="A62" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E62,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B62" s="3" t="str">
+        <f>IF(MOD(C62,2)=1,"Odd (Jul-Nov "&amp;LEFT(A62,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A62,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C62" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E62,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D62" s="2" t="s">
-        <v>208</v>
+      <c r="D62" s="3" t="str">
+        <f>(LEFT(A62,4)-INT((C62-1)/2))&amp;"-"&amp;RIGHT(LEFT(A62,4)-INT((C62-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>127</v>
@@ -23616,8 +23968,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E62,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I62" s="2" t="s">
-        <v>54</v>
+      <c r="I62" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E62,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F019</v>
       </c>
       <c r="J62" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I62,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23658,22 +24011,27 @@
         <f>N62*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T62" s="2" t="s">
-        <v>1196</v>
+      <c r="T62" s="3" t="str">
+        <f>IF(MOD(C62,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="63" spans="1:20">
-      <c r="A63" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C63" s="2">
+      <c r="A63" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E63,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B63" s="3" t="str">
+        <f>IF(MOD(C63,2)=1,"Odd (Jul-Nov "&amp;LEFT(A63,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A63,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C63" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E63,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D63" s="2" t="s">
-        <v>208</v>
+      <c r="D63" s="3" t="str">
+        <f>(LEFT(A63,4)-INT((C63-1)/2))&amp;"-"&amp;RIGHT(LEFT(A63,4)-INT((C63-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>127</v>
@@ -23690,8 +24048,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E63,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I63" s="2" t="s">
-        <v>54</v>
+      <c r="I63" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E63,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F019</v>
       </c>
       <c r="J63" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I63,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23732,22 +24091,27 @@
         <f>N63*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T63" s="2" t="s">
-        <v>1196</v>
+      <c r="T63" s="3" t="str">
+        <f>IF(MOD(C63,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="64" spans="1:20">
-      <c r="A64" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C64" s="2">
+      <c r="A64" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E64,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B64" s="3" t="str">
+        <f>IF(MOD(C64,2)=1,"Odd (Jul-Nov "&amp;LEFT(A64,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A64,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C64" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E64,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D64" s="2" t="s">
-        <v>208</v>
+      <c r="D64" s="3" t="str">
+        <f>(LEFT(A64,4)-INT((C64-1)/2))&amp;"-"&amp;RIGHT(LEFT(A64,4)-INT((C64-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>129</v>
@@ -23764,8 +24128,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E64,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I64" s="2" t="s">
-        <v>71</v>
+      <c r="I64" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E64,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F012</v>
       </c>
       <c r="J64" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I64,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23806,22 +24171,27 @@
         <f>N64*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T64" s="2" t="s">
-        <v>1196</v>
+      <c r="T64" s="3" t="str">
+        <f>IF(MOD(C64,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="65" spans="1:20">
-      <c r="A65" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C65" s="2">
+      <c r="A65" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E65,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B65" s="3" t="str">
+        <f>IF(MOD(C65,2)=1,"Odd (Jul-Nov "&amp;LEFT(A65,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A65,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C65" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E65,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D65" s="2" t="s">
-        <v>208</v>
+      <c r="D65" s="3" t="str">
+        <f>(LEFT(A65,4)-INT((C65-1)/2))&amp;"-"&amp;RIGHT(LEFT(A65,4)-INT((C65-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>129</v>
@@ -23838,8 +24208,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E65,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I65" s="2" t="s">
-        <v>71</v>
+      <c r="I65" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E65,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F012</v>
       </c>
       <c r="J65" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I65,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23880,22 +24251,27 @@
         <f>N65*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T65" s="2" t="s">
-        <v>1196</v>
+      <c r="T65" s="3" t="str">
+        <f>IF(MOD(C65,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="66" spans="1:20">
-      <c r="A66" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C66" s="2">
+      <c r="A66" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E66,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B66" s="3" t="str">
+        <f>IF(MOD(C66,2)=1,"Odd (Jul-Nov "&amp;LEFT(A66,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A66,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C66" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E66,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D66" s="2" t="s">
-        <v>208</v>
+      <c r="D66" s="3" t="str">
+        <f>(LEFT(A66,4)-INT((C66-1)/2))&amp;"-"&amp;RIGHT(LEFT(A66,4)-INT((C66-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>131</v>
@@ -23912,8 +24288,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E66,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I66" s="2" t="s">
-        <v>84</v>
+      <c r="I66" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E66,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F017</v>
       </c>
       <c r="J66" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I66,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -23954,22 +24331,27 @@
         <f>N66*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T66" s="2" t="s">
-        <v>1196</v>
+      <c r="T66" s="3" t="str">
+        <f>IF(MOD(C66,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="67" spans="1:20">
-      <c r="A67" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C67" s="2">
+      <c r="A67" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E67,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B67" s="3" t="str">
+        <f>IF(MOD(C67,2)=1,"Odd (Jul-Nov "&amp;LEFT(A67,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A67,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C67" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E67,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D67" s="2" t="s">
-        <v>208</v>
+      <c r="D67" s="3" t="str">
+        <f>(LEFT(A67,4)-INT((C67-1)/2))&amp;"-"&amp;RIGHT(LEFT(A67,4)-INT((C67-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>131</v>
@@ -23986,8 +24368,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E67,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I67" s="2" t="s">
-        <v>84</v>
+      <c r="I67" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E67,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F017</v>
       </c>
       <c r="J67" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I67,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24028,22 +24411,27 @@
         <f>N67*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T67" s="2" t="s">
-        <v>1196</v>
+      <c r="T67" s="3" t="str">
+        <f>IF(MOD(C67,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="68" spans="1:20">
-      <c r="A68" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C68" s="2">
+      <c r="A68" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E68,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B68" s="3" t="str">
+        <f>IF(MOD(C68,2)=1,"Odd (Jul-Nov "&amp;LEFT(A68,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A68,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C68" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E68,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>208</v>
+      <c r="D68" s="3" t="str">
+        <f>(LEFT(A68,4)-INT((C68-1)/2))&amp;"-"&amp;RIGHT(LEFT(A68,4)-INT((C68-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>133</v>
@@ -24060,8 +24448,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E68,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I68" s="2" t="s">
-        <v>78</v>
+      <c r="I68" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E68,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F003</v>
       </c>
       <c r="J68" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I68,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24102,22 +24491,27 @@
         <f>N68*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T68" s="2" t="s">
-        <v>1196</v>
+      <c r="T68" s="3" t="str">
+        <f>IF(MOD(C68,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="69" spans="1:20">
-      <c r="A69" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C69" s="2">
+      <c r="A69" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E69,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B69" s="3" t="str">
+        <f>IF(MOD(C69,2)=1,"Odd (Jul-Nov "&amp;LEFT(A69,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A69,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C69" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E69,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D69" s="2" t="s">
-        <v>208</v>
+      <c r="D69" s="3" t="str">
+        <f>(LEFT(A69,4)-INT((C69-1)/2))&amp;"-"&amp;RIGHT(LEFT(A69,4)-INT((C69-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>135</v>
@@ -24134,8 +24528,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E69,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I69" s="2" t="s">
-        <v>108</v>
+      <c r="I69" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E69,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F009</v>
       </c>
       <c r="J69" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I69,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24176,22 +24571,27 @@
         <f>N69*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T69" s="2" t="s">
-        <v>1196</v>
+      <c r="T69" s="3" t="str">
+        <f>IF(MOD(C69,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="70" spans="1:20">
-      <c r="A70" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C70" s="2">
+      <c r="A70" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E70,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B70" s="3" t="str">
+        <f>IF(MOD(C70,2)=1,"Odd (Jul-Nov "&amp;LEFT(A70,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A70,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C70" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E70,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>208</v>
+      <c r="D70" s="3" t="str">
+        <f>(LEFT(A70,4)-INT((C70-1)/2))&amp;"-"&amp;RIGHT(LEFT(A70,4)-INT((C70-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>137</v>
@@ -24208,8 +24608,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E70,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I70" s="2" t="s">
-        <v>81</v>
+      <c r="I70" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E70,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F002</v>
       </c>
       <c r="J70" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I70,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24250,22 +24651,27 @@
         <f>N70*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T70" s="2" t="s">
-        <v>1196</v>
+      <c r="T70" s="3" t="str">
+        <f>IF(MOD(C70,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="71" spans="1:20">
-      <c r="A71" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C71" s="2">
+      <c r="A71" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E71,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B71" s="3" t="str">
+        <f>IF(MOD(C71,2)=1,"Odd (Jul-Nov "&amp;LEFT(A71,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A71,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C71" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E71,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>208</v>
+      <c r="D71" s="3" t="str">
+        <f>(LEFT(A71,4)-INT((C71-1)/2))&amp;"-"&amp;RIGHT(LEFT(A71,4)-INT((C71-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>140</v>
@@ -24282,8 +24688,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E71,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I71" s="2" t="s">
-        <v>35</v>
+      <c r="I71" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E71,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F007</v>
       </c>
       <c r="J71" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I71,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24324,22 +24731,27 @@
         <f>N71*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T71" s="2" t="s">
-        <v>1196</v>
+      <c r="T71" s="3" t="str">
+        <f>IF(MOD(C71,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="72" spans="1:20">
-      <c r="A72" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C72" s="2">
+      <c r="A72" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E72,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B72" s="3" t="str">
+        <f>IF(MOD(C72,2)=1,"Odd (Jul-Nov "&amp;LEFT(A72,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A72,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C72" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E72,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D72" s="2" t="s">
-        <v>208</v>
+      <c r="D72" s="3" t="str">
+        <f>(LEFT(A72,4)-INT((C72-1)/2))&amp;"-"&amp;RIGHT(LEFT(A72,4)-INT((C72-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>142</v>
@@ -24356,8 +24768,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E72,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I72" s="2" t="s">
-        <v>58</v>
+      <c r="I72" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E72,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F005</v>
       </c>
       <c r="J72" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I72,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24398,22 +24811,27 @@
         <f>N72*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T72" s="2" t="s">
-        <v>1196</v>
+      <c r="T72" s="3" t="str">
+        <f>IF(MOD(C72,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="73" spans="1:20">
-      <c r="A73" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C73" s="2">
+      <c r="A73" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E73,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B73" s="3" t="str">
+        <f>IF(MOD(C73,2)=1,"Odd (Jul-Nov "&amp;LEFT(A73,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A73,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C73" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E73,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D73" s="2" t="s">
-        <v>208</v>
+      <c r="D73" s="3" t="str">
+        <f>(LEFT(A73,4)-INT((C73-1)/2))&amp;"-"&amp;RIGHT(LEFT(A73,4)-INT((C73-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>145</v>
@@ -24430,8 +24848,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E73,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I73" s="2" t="s">
-        <v>84</v>
+      <c r="I73" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E73,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F017</v>
       </c>
       <c r="J73" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I73,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24472,22 +24891,27 @@
         <f>N73*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T73" s="2" t="s">
-        <v>1196</v>
+      <c r="T73" s="3" t="str">
+        <f>IF(MOD(C73,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="74" spans="1:20">
-      <c r="A74" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C74" s="2">
+      <c r="A74" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E74,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B74" s="3" t="str">
+        <f>IF(MOD(C74,2)=1,"Odd (Jul-Nov "&amp;LEFT(A74,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A74,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C74" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E74,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D74" s="2" t="s">
-        <v>208</v>
+      <c r="D74" s="3" t="str">
+        <f>(LEFT(A74,4)-INT((C74-1)/2))&amp;"-"&amp;RIGHT(LEFT(A74,4)-INT((C74-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>147</v>
@@ -24504,8 +24928,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E74,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I74" s="2" t="s">
-        <v>118</v>
+      <c r="I74" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E74,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F020</v>
       </c>
       <c r="J74" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I74,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24546,22 +24971,27 @@
         <f>N74*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T74" s="2" t="s">
-        <v>1196</v>
+      <c r="T74" s="3" t="str">
+        <f>IF(MOD(C74,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="75" spans="1:20">
-      <c r="A75" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>1195</v>
-      </c>
-      <c r="C75" s="2">
+      <c r="A75" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E75,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B75" s="3" t="str">
+        <f>IF(MOD(C75,2)=1,"Odd (Jul-Nov "&amp;LEFT(A75,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A75,4)+1)&amp;")")</f>
+        <v>Odd (Jul-Nov 2026)</v>
+      </c>
+      <c r="C75" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E75,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>5</v>
       </c>
-      <c r="D75" s="2" t="s">
-        <v>208</v>
+      <c r="D75" s="3" t="str">
+        <f>(LEFT(A75,4)-INT((C75-1)/2))&amp;"-"&amp;RIGHT(LEFT(A75,4)-INT((C75-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>150</v>
@@ -24578,8 +25008,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E75,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I75" s="2" t="s">
-        <v>49</v>
+      <c r="I75" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E75,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F006</v>
       </c>
       <c r="J75" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I75,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24620,22 +25051,27 @@
         <f>N75*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T75" s="2" t="s">
-        <v>1196</v>
+      <c r="T75" s="3" t="str">
+        <f>IF(MOD(C75,2)=1,"Ongoing","Upcoming")</f>
+        <v>Ongoing</v>
       </c>
     </row>
     <row r="76" spans="1:20">
-      <c r="A76" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C76" s="2">
+      <c r="A76" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E76,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B76" s="3" t="str">
+        <f>IF(MOD(C76,2)=1,"Odd (Jul-Nov "&amp;LEFT(A76,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A76,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C76" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E76,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D76" s="2" t="s">
-        <v>208</v>
+      <c r="D76" s="3" t="str">
+        <f>(LEFT(A76,4)-INT((C76-1)/2))&amp;"-"&amp;RIGHT(LEFT(A76,4)-INT((C76-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>152</v>
@@ -24652,8 +25088,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E76,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I76" s="2" t="s">
-        <v>27</v>
+      <c r="I76" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E76,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F018</v>
       </c>
       <c r="J76" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I76,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24694,22 +25131,27 @@
         <f>N76*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T76" s="2" t="s">
-        <v>1198</v>
+      <c r="T76" s="3" t="str">
+        <f>IF(MOD(C76,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="77" spans="1:20">
-      <c r="A77" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C77" s="2">
+      <c r="A77" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E77,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B77" s="3" t="str">
+        <f>IF(MOD(C77,2)=1,"Odd (Jul-Nov "&amp;LEFT(A77,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A77,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C77" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E77,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D77" s="2" t="s">
-        <v>208</v>
+      <c r="D77" s="3" t="str">
+        <f>(LEFT(A77,4)-INT((C77-1)/2))&amp;"-"&amp;RIGHT(LEFT(A77,4)-INT((C77-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>152</v>
@@ -24726,8 +25168,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E77,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I77" s="2" t="s">
-        <v>27</v>
+      <c r="I77" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E77,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F018</v>
       </c>
       <c r="J77" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I77,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24768,22 +25211,27 @@
         <f>N77*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T77" s="2" t="s">
-        <v>1198</v>
+      <c r="T77" s="3" t="str">
+        <f>IF(MOD(C77,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="78" spans="1:20">
-      <c r="A78" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C78" s="2">
+      <c r="A78" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E78,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B78" s="3" t="str">
+        <f>IF(MOD(C78,2)=1,"Odd (Jul-Nov "&amp;LEFT(A78,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A78,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C78" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E78,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D78" s="2" t="s">
-        <v>208</v>
+      <c r="D78" s="3" t="str">
+        <f>(LEFT(A78,4)-INT((C78-1)/2))&amp;"-"&amp;RIGHT(LEFT(A78,4)-INT((C78-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>154</v>
@@ -24800,8 +25248,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E78,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I78" s="2" t="s">
-        <v>64</v>
+      <c r="I78" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E78,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F014</v>
       </c>
       <c r="J78" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I78,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24842,22 +25291,27 @@
         <f>N78*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T78" s="2" t="s">
-        <v>1198</v>
+      <c r="T78" s="3" t="str">
+        <f>IF(MOD(C78,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="79" spans="1:20">
-      <c r="A79" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C79" s="2">
+      <c r="A79" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E79,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B79" s="3" t="str">
+        <f>IF(MOD(C79,2)=1,"Odd (Jul-Nov "&amp;LEFT(A79,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A79,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C79" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E79,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D79" s="2" t="s">
-        <v>208</v>
+      <c r="D79" s="3" t="str">
+        <f>(LEFT(A79,4)-INT((C79-1)/2))&amp;"-"&amp;RIGHT(LEFT(A79,4)-INT((C79-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>154</v>
@@ -24874,8 +25328,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E79,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I79" s="2" t="s">
-        <v>64</v>
+      <c r="I79" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E79,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F014</v>
       </c>
       <c r="J79" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I79,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24916,22 +25371,27 @@
         <f>N79*FacultyCreditHoursPerCredit</f>
         <v>45</v>
       </c>
-      <c r="T79" s="2" t="s">
-        <v>1198</v>
+      <c r="T79" s="3" t="str">
+        <f>IF(MOD(C79,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="80" spans="1:20">
-      <c r="A80" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C80" s="2">
+      <c r="A80" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E80,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B80" s="3" t="str">
+        <f>IF(MOD(C80,2)=1,"Odd (Jul-Nov "&amp;LEFT(A80,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A80,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C80" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E80,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D80" s="2" t="s">
-        <v>208</v>
+      <c r="D80" s="3" t="str">
+        <f>(LEFT(A80,4)-INT((C80-1)/2))&amp;"-"&amp;RIGHT(LEFT(A80,4)-INT((C80-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>156</v>
@@ -24948,8 +25408,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E80,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I80" s="2" t="s">
-        <v>126</v>
+      <c r="I80" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E80,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F001</v>
       </c>
       <c r="J80" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I80,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -24990,22 +25451,27 @@
         <f>N80*FacultyCreditHoursPerCredit</f>
         <v>90</v>
       </c>
-      <c r="T80" s="2" t="s">
-        <v>1198</v>
+      <c r="T80" s="3" t="str">
+        <f>IF(MOD(C80,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="81" spans="1:20">
-      <c r="A81" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C81" s="2">
+      <c r="A81" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E81,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B81" s="3" t="str">
+        <f>IF(MOD(C81,2)=1,"Odd (Jul-Nov "&amp;LEFT(A81,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A81,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C81" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E81,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D81" s="2" t="s">
-        <v>208</v>
+      <c r="D81" s="3" t="str">
+        <f>(LEFT(A81,4)-INT((C81-1)/2))&amp;"-"&amp;RIGHT(LEFT(A81,4)-INT((C81-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>156</v>
@@ -25022,8 +25488,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E81,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I81" s="2" t="s">
-        <v>126</v>
+      <c r="I81" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E81,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F001</v>
       </c>
       <c r="J81" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I81,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25064,22 +25531,27 @@
         <f>N81*FacultyCreditHoursPerCredit</f>
         <v>90</v>
       </c>
-      <c r="T81" s="2" t="s">
-        <v>1198</v>
+      <c r="T81" s="3" t="str">
+        <f>IF(MOD(C81,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="82" spans="1:20">
-      <c r="A82" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C82" s="2">
+      <c r="A82" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E82,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B82" s="3" t="str">
+        <f>IF(MOD(C82,2)=1,"Odd (Jul-Nov "&amp;LEFT(A82,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A82,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C82" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E82,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D82" s="2" t="s">
-        <v>208</v>
+      <c r="D82" s="3" t="str">
+        <f>(LEFT(A82,4)-INT((C82-1)/2))&amp;"-"&amp;RIGHT(LEFT(A82,4)-INT((C82-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>158</v>
@@ -25096,8 +25568,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E82,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I82" s="2" t="s">
-        <v>71</v>
+      <c r="I82" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E82,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F012</v>
       </c>
       <c r="J82" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I82,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25138,22 +25611,27 @@
         <f>N82*FacultyCreditHoursPerCredit</f>
         <v>15</v>
       </c>
-      <c r="T82" s="2" t="s">
-        <v>1198</v>
+      <c r="T82" s="3" t="str">
+        <f>IF(MOD(C82,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="83" spans="1:20">
-      <c r="A83" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C83" s="2">
+      <c r="A83" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E83,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B83" s="3" t="str">
+        <f>IF(MOD(C83,2)=1,"Odd (Jul-Nov "&amp;LEFT(A83,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A83,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C83" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E83,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D83" s="2" t="s">
-        <v>208</v>
+      <c r="D83" s="3" t="str">
+        <f>(LEFT(A83,4)-INT((C83-1)/2))&amp;"-"&amp;RIGHT(LEFT(A83,4)-INT((C83-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>158</v>
@@ -25170,8 +25648,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E83,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Core</v>
       </c>
-      <c r="I83" s="2" t="s">
-        <v>71</v>
+      <c r="I83" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E83,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F012</v>
       </c>
       <c r="J83" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I83,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25212,22 +25691,27 @@
         <f>N83*FacultyCreditHoursPerCredit</f>
         <v>15</v>
       </c>
-      <c r="T83" s="2" t="s">
-        <v>1198</v>
+      <c r="T83" s="3" t="str">
+        <f>IF(MOD(C83,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="84" spans="1:20">
-      <c r="A84" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C84" s="2">
+      <c r="A84" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E84,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B84" s="3" t="str">
+        <f>IF(MOD(C84,2)=1,"Odd (Jul-Nov "&amp;LEFT(A84,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A84,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C84" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E84,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D84" s="2" t="s">
-        <v>208</v>
+      <c r="D84" s="3" t="str">
+        <f>(LEFT(A84,4)-INT((C84-1)/2))&amp;"-"&amp;RIGHT(LEFT(A84,4)-INT((C84-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>160</v>
@@ -25244,8 +25728,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E84,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I84" s="2" t="s">
-        <v>118</v>
+      <c r="I84" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E84,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F020</v>
       </c>
       <c r="J84" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I84,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25286,22 +25771,27 @@
         <f>N84*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T84" s="2" t="s">
-        <v>1198</v>
+      <c r="T84" s="3" t="str">
+        <f>IF(MOD(C84,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="85" spans="1:20">
-      <c r="A85" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C85" s="2">
+      <c r="A85" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E85,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B85" s="3" t="str">
+        <f>IF(MOD(C85,2)=1,"Odd (Jul-Nov "&amp;LEFT(A85,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A85,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C85" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E85,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D85" s="2" t="s">
-        <v>208</v>
+      <c r="D85" s="3" t="str">
+        <f>(LEFT(A85,4)-INT((C85-1)/2))&amp;"-"&amp;RIGHT(LEFT(A85,4)-INT((C85-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>162</v>
@@ -25318,8 +25808,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E85,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I85" s="2" t="s">
-        <v>108</v>
+      <c r="I85" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E85,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F009</v>
       </c>
       <c r="J85" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I85,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25360,22 +25851,27 @@
         <f>N85*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T85" s="2" t="s">
-        <v>1198</v>
+      <c r="T85" s="3" t="str">
+        <f>IF(MOD(C85,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="86" spans="1:20">
-      <c r="A86" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C86" s="2">
+      <c r="A86" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E86,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B86" s="3" t="str">
+        <f>IF(MOD(C86,2)=1,"Odd (Jul-Nov "&amp;LEFT(A86,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A86,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C86" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E86,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D86" s="2" t="s">
-        <v>208</v>
+      <c r="D86" s="3" t="str">
+        <f>(LEFT(A86,4)-INT((C86-1)/2))&amp;"-"&amp;RIGHT(LEFT(A86,4)-INT((C86-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>164</v>
@@ -25392,8 +25888,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E86,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I86" s="2" t="s">
-        <v>81</v>
+      <c r="I86" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E86,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F002</v>
       </c>
       <c r="J86" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I86,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25434,22 +25931,27 @@
         <f>N86*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T86" s="2" t="s">
-        <v>1198</v>
+      <c r="T86" s="3" t="str">
+        <f>IF(MOD(C86,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="87" spans="1:20">
-      <c r="A87" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C87" s="2">
+      <c r="A87" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E87,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B87" s="3" t="str">
+        <f>IF(MOD(C87,2)=1,"Odd (Jul-Nov "&amp;LEFT(A87,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A87,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C87" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E87,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D87" s="2" t="s">
-        <v>208</v>
+      <c r="D87" s="3" t="str">
+        <f>(LEFT(A87,4)-INT((C87-1)/2))&amp;"-"&amp;RIGHT(LEFT(A87,4)-INT((C87-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>166</v>
@@ -25466,8 +25968,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E87,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I87" s="2" t="s">
-        <v>35</v>
+      <c r="I87" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E87,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F007</v>
       </c>
       <c r="J87" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I87,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25508,22 +26011,27 @@
         <f>N87*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T87" s="2" t="s">
-        <v>1198</v>
+      <c r="T87" s="3" t="str">
+        <f>IF(MOD(C87,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="88" spans="1:20">
-      <c r="A88" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C88" s="2">
+      <c r="A88" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E88,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B88" s="3" t="str">
+        <f>IF(MOD(C88,2)=1,"Odd (Jul-Nov "&amp;LEFT(A88,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A88,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C88" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E88,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D88" s="2" t="s">
-        <v>208</v>
+      <c r="D88" s="3" t="str">
+        <f>(LEFT(A88,4)-INT((C88-1)/2))&amp;"-"&amp;RIGHT(LEFT(A88,4)-INT((C88-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>168</v>
@@ -25540,8 +26048,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E88,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I88" s="2" t="s">
-        <v>58</v>
+      <c r="I88" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E88,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F005</v>
       </c>
       <c r="J88" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I88,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25582,22 +26091,27 @@
         <f>N88*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T88" s="2" t="s">
-        <v>1198</v>
+      <c r="T88" s="3" t="str">
+        <f>IF(MOD(C88,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="89" spans="1:20">
-      <c r="A89" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C89" s="2">
+      <c r="A89" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E89,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B89" s="3" t="str">
+        <f>IF(MOD(C89,2)=1,"Odd (Jul-Nov "&amp;LEFT(A89,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A89,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C89" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E89,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D89" s="2" t="s">
-        <v>208</v>
+      <c r="D89" s="3" t="str">
+        <f>(LEFT(A89,4)-INT((C89-1)/2))&amp;"-"&amp;RIGHT(LEFT(A89,4)-INT((C89-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>170</v>
@@ -25614,8 +26128,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E89,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I89" s="2" t="s">
-        <v>87</v>
+      <c r="I89" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E89,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F010</v>
       </c>
       <c r="J89" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I89,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25656,22 +26171,27 @@
         <f>N89*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T89" s="2" t="s">
-        <v>1198</v>
+      <c r="T89" s="3" t="str">
+        <f>IF(MOD(C89,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="90" spans="1:20">
-      <c r="A90" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C90" s="2">
+      <c r="A90" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E90,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B90" s="3" t="str">
+        <f>IF(MOD(C90,2)=1,"Odd (Jul-Nov "&amp;LEFT(A90,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A90,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C90" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E90,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D90" s="2" t="s">
-        <v>208</v>
+      <c r="D90" s="3" t="str">
+        <f>(LEFT(A90,4)-INT((C90-1)/2))&amp;"-"&amp;RIGHT(LEFT(A90,4)-INT((C90-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>172</v>
@@ -25688,8 +26208,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E90,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I90" s="2" t="s">
-        <v>39</v>
+      <c r="I90" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E90,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F013</v>
       </c>
       <c r="J90" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I90,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25730,22 +26251,27 @@
         <f>N90*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T90" s="2" t="s">
-        <v>1198</v>
+      <c r="T90" s="3" t="str">
+        <f>IF(MOD(C90,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
     <row r="91" spans="1:20">
-      <c r="A91" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B91" s="2" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C91" s="2">
+      <c r="A91" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$A$2:$A$57,MATCH(E91,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>2026-27</v>
+      </c>
+      <c r="B91" s="3" t="str">
+        <f>IF(MOD(C91,2)=1,"Odd (Jul-Nov "&amp;LEFT(A91,4)&amp;")","Even (Jan-Apr "&amp;(LEFT(A91,4)+1)&amp;")")</f>
+        <v>Even (Jan-Apr 2027)</v>
+      </c>
+      <c r="C91" s="3">
+        <f>INDEX('Curriculum Master'!$C$2:$C$57,MATCH(E91,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>6</v>
       </c>
-      <c r="D91" s="2" t="s">
-        <v>208</v>
+      <c r="D91" s="3" t="str">
+        <f>(LEFT(A91,4)-INT((C91-1)/2))&amp;"-"&amp;RIGHT(LEFT(A91,4)-INT((C91-1)/2)+3,2)</f>
+        <v>2024-27</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>174</v>
@@ -25762,8 +26288,9 @@
         <f>INDEX('Curriculum Master'!$N$2:$N$57,MATCH(E91,'Curriculum Master'!$D$2:$D$57,0))</f>
         <v>Elective</v>
       </c>
-      <c r="I91" s="2" t="s">
-        <v>49</v>
+      <c r="I91" s="3" t="str">
+        <f>INDEX('Curriculum Master'!$R$2:$R$57,MATCH(E91,'Curriculum Master'!$D$2:$D$57,0))</f>
+        <v>F006</v>
       </c>
       <c r="J91" s="3" t="str">
         <f>INDEX('Faculty Master'!$B$2:$B$21,MATCH(I91,'Faculty Master'!$A$2:$A$21,0))</f>
@@ -25804,8 +26331,9 @@
         <f>N91*FacultyCreditHoursPerCredit</f>
         <v>60</v>
       </c>
-      <c r="T91" s="2" t="s">
-        <v>1198</v>
+      <c r="T91" s="3" t="str">
+        <f>IF(MOD(C91,2)=1,"Ongoing","Upcoming")</f>
+        <v>Upcoming</v>
       </c>
     </row>
   </sheetData>
@@ -25829,57 +26357,57 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>1199</v>
+        <v>1195</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1200</v>
+        <v>1196</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1201</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>1202</v>
+        <v>1198</v>
       </c>
       <c r="B2" s="2">
         <v>10</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1203</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>1204</v>
+        <v>1200</v>
       </c>
       <c r="B3" s="2">
         <v>75</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1205</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>1206</v>
+        <v>1202</v>
       </c>
       <c r="B4" s="2">
         <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1207</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>1208</v>
+        <v>1204</v>
       </c>
       <c r="B5" s="2">
         <v>150</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1209</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -25892,12 +26420,12 @@
         <v>12.5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1210</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="4" t="s">
-        <v>1211</v>
+        <v>1207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>